<commit_message>
Updating workflow mapping and the scripts for merging historical sources
</commit_message>
<xml_diff>
--- a/documentation/workflow/bc_bronze_workflow_mapping.xlsx
+++ b/documentation/workflow/bc_bronze_workflow_mapping.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11109"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fantasysuperkick/workspace/ccg/datawarehouse/documentation/workflow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC916EC9-D8CB-3F49-B18B-AB80085D7161}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDCD3F2D-7D31-EE4B-8F4C-A62A3958230E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="660" yWindow="500" windowWidth="28140" windowHeight="17500" xr2:uid="{2F7A961D-90EA-0F4A-9BBB-FA6BCAC4A400}"/>
   </bookViews>
@@ -1662,9 +1662,6 @@
     <t>locationcode, bincode, variantcode, unitofmeasurecode</t>
   </si>
   <si>
-    <t>cuurencycode</t>
-  </si>
-  <si>
     <t>tableid</t>
   </si>
   <si>
@@ -1702,6 +1699,9 @@
   </si>
   <si>
     <t>worksheetbatchname</t>
+  </si>
+  <si>
+    <t>currencycode, company, source_system</t>
   </si>
 </sst>
 </file>
@@ -2875,10 +2875,10 @@
         <v>112</v>
       </c>
       <c r="C49" t="s">
-        <v>540</v>
+        <v>113</v>
       </c>
       <c r="D49" t="s">
-        <v>10</v>
+        <v>553</v>
       </c>
       <c r="E49" t="s">
         <v>113</v>
@@ -3047,7 +3047,7 @@
         <v>131</v>
       </c>
       <c r="C60" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="D60" t="s">
         <v>10</v>
@@ -3162,7 +3162,7 @@
         <v>143</v>
       </c>
       <c r="C68" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="D68" t="s">
         <v>10</v>
@@ -3193,7 +3193,7 @@
         <v>147</v>
       </c>
       <c r="C70" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="D70" t="s">
         <v>10</v>
@@ -3480,7 +3480,7 @@
         <v>178</v>
       </c>
       <c r="C89" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="D89" t="s">
         <v>10</v>
@@ -3748,7 +3748,7 @@
         <v>204</v>
       </c>
       <c r="C106" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="D106" t="s">
         <v>10</v>
@@ -3869,7 +3869,7 @@
         <v>214</v>
       </c>
       <c r="C114" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="D114" t="s">
         <v>10</v>
@@ -4053,7 +4053,7 @@
         <v>10</v>
       </c>
       <c r="E125" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="F125" t="s">
         <v>520</v>
@@ -4202,7 +4202,7 @@
         <v>246</v>
       </c>
       <c r="C135" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="D135" t="s">
         <v>10</v>
@@ -4599,7 +4599,7 @@
         <v>10</v>
       </c>
       <c r="E161" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="F161" t="s">
         <v>520</v>
@@ -5303,7 +5303,7 @@
         <v>10</v>
       </c>
       <c r="E204" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="F204" t="s">
         <v>520</v>
@@ -5410,7 +5410,7 @@
         <v>384</v>
       </c>
       <c r="C211" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="D211" t="s">
         <v>10</v>
@@ -5822,7 +5822,7 @@
         <v>427</v>
       </c>
       <c r="C237" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="D237" t="s">
         <v>10</v>
@@ -6189,7 +6189,7 @@
         <v>10</v>
       </c>
       <c r="E260" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="F260" t="s">
         <v>520</v>
@@ -6346,7 +6346,7 @@
         <v>476</v>
       </c>
       <c r="C271" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="D271" t="s">
         <v>10</v>
@@ -6543,7 +6543,7 @@
         <v>496</v>
       </c>
       <c r="C284" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="D284" t="s">
         <v>10</v>

</xml_diff>

<commit_message>
update for partition key
</commit_message>
<xml_diff>
--- a/documentation/workflow/bc_bronze_workflow_mapping.xlsx
+++ b/documentation/workflow/bc_bronze_workflow_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fantasysuperkick/workspace/ccg/datawarehouse/documentation/workflow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDCD3F2D-7D31-EE4B-8F4C-A62A3958230E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5DB48FA-FF6F-0340-8BAB-DA1E53BF69DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="660" yWindow="500" windowWidth="28140" windowHeight="17500" xr2:uid="{2F7A961D-90EA-0F4A-9BBB-FA6BCAC4A400}"/>
   </bookViews>
@@ -3695,7 +3695,7 @@
         <v>198</v>
       </c>
       <c r="F102" t="s">
-        <v>520</v>
+        <v>522</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
update for ostendo pipeline
</commit_message>
<xml_diff>
--- a/documentation/workflow/bc_bronze_workflow_mapping.xlsx
+++ b/documentation/workflow/bc_bronze_workflow_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fantasysuperkick/workspace/ccg/datawarehouse/documentation/workflow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5DB48FA-FF6F-0340-8BAB-DA1E53BF69DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{861A0259-3088-4C4C-9F49-0FD9BAAE4F9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="660" yWindow="500" windowWidth="28140" windowHeight="17500" xr2:uid="{2F7A961D-90EA-0F4A-9BBB-FA6BCAC4A400}"/>
   </bookViews>
@@ -19,7 +19,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$C$1:$C$299</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -3909,7 +3909,7 @@
         <v>220</v>
       </c>
       <c r="F116" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.2">
@@ -4531,7 +4531,7 @@
         <v>17</v>
       </c>
       <c r="D157" t="s">
-        <v>283</v>
+        <v>104</v>
       </c>
       <c r="E157" t="s">
         <v>284</v>

</xml_diff>

<commit_message>
Update BC pipelines for bronze
</commit_message>
<xml_diff>
--- a/documentation/workflow/bc_bronze_workflow_mapping.xlsx
+++ b/documentation/workflow/bc_bronze_workflow_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fantasysuperkick/workspace/ccg/datawarehouse/documentation/workflow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2340E6BF-36C6-1B43-A731-4108F257526C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{571F3020-FD7B-0E48-A440-C51DC1635C26}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="660" yWindow="500" windowWidth="28140" windowHeight="17500" xr2:uid="{2F7A961D-90EA-0F4A-9BBB-FA6BCAC4A400}"/>
   </bookViews>
@@ -1587,9 +1587,6 @@
     <t>glacccategoryentryno, company, source_system</t>
   </si>
   <si>
-    <t>, company, source_system</t>
-  </si>
-  <si>
     <t>startingdate, company, source_system</t>
   </si>
   <si>
@@ -1657,6 +1654,9 @@
   </si>
   <si>
     <t>tableid, company, source_system</t>
+  </si>
+  <si>
+    <t>Bronze_Source_Keys</t>
   </si>
 </sst>
 </file>
@@ -2055,7 +2055,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="22.1640625" customWidth="1"/>
-    <col min="3" max="3" width="30.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="52.83203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="39.1640625" customWidth="1"/>
     <col min="5" max="5" width="49.83203125" customWidth="1"/>
   </cols>
@@ -2068,7 +2068,7 @@
         <v>503</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>515</v>
+        <v>538</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>505</v>
@@ -2133,7 +2133,7 @@
         <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="D5" t="s">
         <v>10</v>
@@ -2147,7 +2147,7 @@
         <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="D6" t="s">
         <v>7</v>
@@ -2311,7 +2311,7 @@
         <v>35</v>
       </c>
       <c r="C16" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="D16" t="s">
         <v>7</v>
@@ -2390,7 +2390,7 @@
         <v>46</v>
       </c>
       <c r="C21" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="D21" t="s">
         <v>7</v>
@@ -2520,7 +2520,7 @@
         <v>61</v>
       </c>
       <c r="C29" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="E29" t="s">
         <v>62</v>
@@ -2568,7 +2568,7 @@
         <v>67</v>
       </c>
       <c r="C32" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="D32" t="s">
         <v>7</v>
@@ -2616,7 +2616,7 @@
         <v>72</v>
       </c>
       <c r="C35" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="D35" t="s">
         <v>7</v>
@@ -2630,7 +2630,7 @@
         <v>73</v>
       </c>
       <c r="C36" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="D36" t="s">
         <v>7</v>
@@ -2760,7 +2760,7 @@
         <v>90</v>
       </c>
       <c r="C44" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="D44" t="s">
         <v>7</v>
@@ -2774,7 +2774,7 @@
         <v>91</v>
       </c>
       <c r="C45" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="D45" t="s">
         <v>7</v>
@@ -2864,7 +2864,7 @@
         <v>98</v>
       </c>
       <c r="C51" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="E51" t="s">
         <v>99</v>
@@ -3002,7 +3002,7 @@
         <v>113</v>
       </c>
       <c r="C60" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="D60" t="s">
         <v>7</v>
@@ -3044,7 +3044,7 @@
         <v>117</v>
       </c>
       <c r="C63" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="F63" t="s">
         <v>493</v>
@@ -3117,7 +3117,7 @@
         <v>124</v>
       </c>
       <c r="C68" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="D68" t="s">
         <v>7</v>
@@ -3148,7 +3148,7 @@
         <v>128</v>
       </c>
       <c r="C70" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="D70" t="s">
         <v>7</v>
@@ -3176,7 +3176,7 @@
         <v>130</v>
       </c>
       <c r="C72" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="D72" t="s">
         <v>17</v>
@@ -3193,7 +3193,7 @@
         <v>132</v>
       </c>
       <c r="C73" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="E73" t="s">
         <v>133</v>
@@ -3207,7 +3207,7 @@
         <v>134</v>
       </c>
       <c r="C74" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="E74" t="s">
         <v>135</v>
@@ -3249,7 +3249,7 @@
         <v>138</v>
       </c>
       <c r="C77" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="D77" t="s">
         <v>7</v>
@@ -3373,7 +3373,7 @@
         <v>151</v>
       </c>
       <c r="C85" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="D85" t="s">
         <v>7</v>
@@ -3435,7 +3435,7 @@
         <v>157</v>
       </c>
       <c r="C89" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="D89" t="s">
         <v>7</v>
@@ -3624,7 +3624,7 @@
         <v>175</v>
       </c>
       <c r="C101" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="D101" t="s">
         <v>7</v>
@@ -3658,7 +3658,7 @@
         <v>178</v>
       </c>
       <c r="C103" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="F103" t="s">
         <v>493</v>
@@ -3703,7 +3703,7 @@
         <v>183</v>
       </c>
       <c r="C106" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="D106" t="s">
         <v>7</v>
@@ -3824,7 +3824,7 @@
         <v>193</v>
       </c>
       <c r="C114" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="D114" t="s">
         <v>7</v>
@@ -3858,7 +3858,7 @@
         <v>197</v>
       </c>
       <c r="C116" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="E116" t="s">
         <v>198</v>
@@ -3872,7 +3872,7 @@
         <v>199</v>
       </c>
       <c r="C117" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="E117" t="s">
         <v>200</v>
@@ -3886,7 +3886,7 @@
         <v>201</v>
       </c>
       <c r="C118" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="D118" t="s">
         <v>17</v>
@@ -4002,7 +4002,7 @@
         <v>212</v>
       </c>
       <c r="C125" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="D125" t="s">
         <v>7</v>
@@ -4157,7 +4157,7 @@
         <v>224</v>
       </c>
       <c r="C135" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="D135" t="s">
         <v>7</v>
@@ -4401,7 +4401,7 @@
         <v>253</v>
       </c>
       <c r="C152" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="D152" t="s">
         <v>7</v>
@@ -4548,7 +4548,7 @@
         <v>267</v>
       </c>
       <c r="C161" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="D161" t="s">
         <v>7</v>
@@ -5125,7 +5125,7 @@
         <v>331</v>
       </c>
       <c r="C196" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="E196" t="s">
         <v>332</v>
@@ -5252,7 +5252,7 @@
         <v>347</v>
       </c>
       <c r="C204" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="D204" t="s">
         <v>7</v>
@@ -5365,7 +5365,7 @@
         <v>358</v>
       </c>
       <c r="C211" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="D211" t="s">
         <v>7</v>
@@ -5777,7 +5777,7 @@
         <v>401</v>
       </c>
       <c r="C237" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="D237" t="s">
         <v>7</v>
@@ -6138,7 +6138,7 @@
         <v>434</v>
       </c>
       <c r="C260" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="D260" t="s">
         <v>7</v>
@@ -6301,7 +6301,7 @@
         <v>450</v>
       </c>
       <c r="C271" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="D271" t="s">
         <v>7</v>
@@ -6363,7 +6363,7 @@
         <v>456</v>
       </c>
       <c r="C275" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="E275" t="s">
         <v>457</v>
@@ -6498,7 +6498,7 @@
         <v>469</v>
       </c>
       <c r="C284" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="D284" t="s">
         <v>7</v>
@@ -6766,7 +6766,6 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="C1:C299" xr:uid="{4E95DFF8-97A2-F246-A8EF-BFAEB7CC069C}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>

</xml_diff>

<commit_message>
update for workflow mapping
</commit_message>
<xml_diff>
--- a/documentation/workflow/bc_bronze_workflow_mapping.xlsx
+++ b/documentation/workflow/bc_bronze_workflow_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fantasysuperkick/workspace/ccg/datawarehouse/documentation/workflow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4D219AB-F1AC-944D-9384-3BC2D8463417}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D1FE482-DB01-6B44-803F-FD1DD29D4B07}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="660" yWindow="500" windowWidth="28140" windowHeight="17500" xr2:uid="{2F7A961D-90EA-0F4A-9BBB-FA6BCAC4A400}"/>
   </bookViews>
@@ -1665,10 +1665,10 @@
     <t>dimensionsetid,dimensioncode</t>
   </si>
   <si>
-    <t>dimensionvaluecode</t>
-  </si>
-  <si>
     <t>dimensionsetid,dimensioncode,company,source_system</t>
+  </si>
+  <si>
+    <t>dimensionvaluecode,shortcutdimensionno</t>
   </si>
 </sst>
 </file>
@@ -6785,10 +6785,10 @@
         <v>540</v>
       </c>
       <c r="D300" t="s">
+        <v>541</v>
+      </c>
+      <c r="E300" t="s">
         <v>542</v>
-      </c>
-      <c r="E300" t="s">
-        <v>541</v>
       </c>
       <c r="F300" t="s">
         <v>493</v>

</xml_diff>

<commit_message>
Update BC Bronze workflow mapping Excel files
</commit_message>
<xml_diff>
--- a/documentation/workflow/bc_bronze_workflow_mapping.xlsx
+++ b/documentation/workflow/bc_bronze_workflow_mapping.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\Exco_Partners\Data-Warehouse\documentation\workflow\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE1A3522-FFFB-439C-B386-5EA607415156}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7BE18F8-C239-46F3-BD3C-F5AB1F157FD2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2F7A961D-90EA-0F4A-9BBB-FA6BCAC4A400}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1433" uniqueCount="559">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1426" uniqueCount="552">
   <si>
     <t>3PLHeader</t>
   </si>
@@ -1659,40 +1659,19 @@
     <t>Bronze_Source_Keys</t>
   </si>
   <si>
-    <t>segmentno, segmentactionno, segmentlineno</t>
-  </si>
-  <si>
     <t>segmentno, segmentactionno, segmentlineno, company, source_system</t>
   </si>
   <si>
-    <t>transferfromcode, transfertocode</t>
-  </si>
-  <si>
     <t>transferfromcode, transfertocode, company, source_system</t>
   </si>
   <si>
-    <t>valueentryno</t>
-  </si>
-  <si>
     <t>valueentryno, company, source_system</t>
   </si>
   <si>
-    <t>sourcetype, sourcsSubtype, sourceno,  locationcode, type</t>
-  </si>
-  <si>
     <t>sourcetype, sourcsSubtype, sourceno,  locationcode, type, company, source_system</t>
   </si>
   <si>
-    <t>sourcetype, sourcecode, basecalendarcode, sourcename</t>
-  </si>
-  <si>
     <t>sourcetype, sourcecode, basecalendarcode, sourcename, company, source_system</t>
-  </si>
-  <si>
-    <t>itementryno</t>
-  </si>
-  <si>
-    <t>daynumber</t>
   </si>
   <si>
     <t>daynumber, company, source_system</t>
@@ -2115,7 +2094,7 @@
   <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6"/>
   <cols>
     <col min="1" max="2" width="22.19921875" customWidth="1"/>
-    <col min="3" max="3" width="52.796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="72.09765625" customWidth="1"/>
     <col min="4" max="4" width="59.59765625" customWidth="1"/>
     <col min="5" max="5" width="49.796875" customWidth="1"/>
     <col min="6" max="6" width="20.59765625" customWidth="1"/>
@@ -6828,27 +6807,21 @@
     </row>
     <row r="300" spans="1:6">
       <c r="A300" t="s">
-        <v>558</v>
+        <v>551</v>
       </c>
       <c r="C300" t="s">
         <v>539</v>
       </c>
-      <c r="D300" t="s">
-        <v>540</v>
-      </c>
       <c r="F300" t="s">
         <v>493</v>
       </c>
     </row>
     <row r="301" spans="1:6">
       <c r="A301" t="s">
-        <v>557</v>
+        <v>550</v>
       </c>
       <c r="C301" t="s">
-        <v>541</v>
-      </c>
-      <c r="D301" t="s">
-        <v>542</v>
+        <v>540</v>
       </c>
       <c r="F301" t="s">
         <v>493</v>
@@ -6856,13 +6829,10 @@
     </row>
     <row r="302" spans="1:6">
       <c r="A302" t="s">
-        <v>556</v>
+        <v>549</v>
       </c>
       <c r="C302" t="s">
-        <v>543</v>
-      </c>
-      <c r="D302" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="F302" t="s">
         <v>493</v>
@@ -6870,13 +6840,10 @@
     </row>
     <row r="303" spans="1:6">
       <c r="A303" t="s">
-        <v>555</v>
+        <v>548</v>
       </c>
       <c r="C303" t="s">
-        <v>545</v>
-      </c>
-      <c r="D303" t="s">
-        <v>546</v>
+        <v>542</v>
       </c>
       <c r="F303" t="s">
         <v>493</v>
@@ -6884,13 +6851,10 @@
     </row>
     <row r="304" spans="1:6">
       <c r="A304" t="s">
-        <v>554</v>
+        <v>547</v>
       </c>
       <c r="C304" t="s">
-        <v>547</v>
-      </c>
-      <c r="D304" t="s">
-        <v>548</v>
+        <v>543</v>
       </c>
       <c r="F304" t="s">
         <v>493</v>
@@ -6898,12 +6862,9 @@
     </row>
     <row r="305" spans="1:6">
       <c r="A305" t="s">
-        <v>553</v>
+        <v>546</v>
       </c>
       <c r="C305" t="s">
-        <v>549</v>
-      </c>
-      <c r="D305" t="s">
         <v>530</v>
       </c>
       <c r="F305" t="s">
@@ -6912,13 +6873,10 @@
     </row>
     <row r="306" spans="1:6">
       <c r="A306" t="s">
-        <v>552</v>
+        <v>545</v>
       </c>
       <c r="C306" t="s">
-        <v>550</v>
-      </c>
-      <c r="D306" t="s">
-        <v>551</v>
+        <v>544</v>
       </c>
       <c r="F306" t="s">
         <v>493</v>

</xml_diff>

<commit_message>
update to include dimensionsetentry
</commit_message>
<xml_diff>
--- a/documentation/workflow/bc_bronze_workflow_mapping.xlsx
+++ b/documentation/workflow/bc_bronze_workflow_mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\Exco_Partners\Data-Warehouse\documentation\workflow\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fantasysuperkick/workspace/ccg/datawarehouse/documentation/workflow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{658935A6-887B-4AB9-BF16-134DC54F4EAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{910E5B33-68BC-0747-B38C-2D1A38332D93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="21220" yWindow="4340" windowWidth="28800" windowHeight="15410" xr2:uid="{2F7A961D-90EA-0F4A-9BBB-FA6BCAC4A400}"/>
+    <workbookView xWindow="660" yWindow="500" windowWidth="23260" windowHeight="12460" xr2:uid="{2F7A961D-90EA-0F4A-9BBB-FA6BCAC4A400}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1426" uniqueCount="552">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1430" uniqueCount="555">
   <si>
     <t>3PLHeader</t>
   </si>
@@ -1695,14 +1695,23 @@
     <t>SegmentHistory</t>
   </si>
   <si>
-    <t>sourcetype, sourcesubtype, sourceno,  locationcode, type, company, source_system</t>
+    <t>DimensionSetEntry</t>
+  </si>
+  <si>
+    <t>sourcetype, sourcessubtype, sourceno,  locationcode, type, company, source_system</t>
+  </si>
+  <si>
+    <t>dimensionsetid, dimensioncode,company, source_system</t>
+  </si>
+  <si>
+    <t>dimensionvaluecode,globaldimensionno</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2090,17 +2099,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E95DFF8-97A2-F246-A8EF-BFAEB7CC069C}">
-  <dimension ref="A1:F306"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6"/>
+  <dimension ref="A1:F307"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="2" width="22.19921875" customWidth="1"/>
-    <col min="3" max="3" width="72.09765625" customWidth="1"/>
-    <col min="4" max="4" width="59.59765625" customWidth="1"/>
-    <col min="5" max="5" width="49.796875" customWidth="1"/>
-    <col min="6" max="6" width="20.59765625" customWidth="1"/>
+    <col min="1" max="2" width="22.1640625" customWidth="1"/>
+    <col min="3" max="3" width="72.1640625" customWidth="1"/>
+    <col min="4" max="4" width="59.6640625" customWidth="1"/>
+    <col min="5" max="5" width="49.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>504</v>
       </c>
@@ -2120,7 +2129,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="2" spans="1:6">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2137,7 +2146,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2154,7 +2163,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="4" spans="1:6">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -2168,7 +2177,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="5" spans="1:6">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2182,7 +2191,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="6" spans="1:6">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -2199,7 +2208,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="7" spans="1:6">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -2213,7 +2222,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="8" spans="1:6">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -2230,7 +2239,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -2244,7 +2253,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="10" spans="1:6">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -2261,7 +2270,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="11" spans="1:6">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -2278,7 +2287,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="12" spans="1:6">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -2295,7 +2304,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="13" spans="1:6">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>26</v>
       </c>
@@ -2312,7 +2321,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="14" spans="1:6">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>28</v>
       </c>
@@ -2329,7 +2338,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="15" spans="1:6">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -2346,7 +2355,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="16" spans="1:6">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>35</v>
       </c>
@@ -2360,7 +2369,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="17" spans="1:6">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>36</v>
       </c>
@@ -2377,7 +2386,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="18" spans="1:6">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>39</v>
       </c>
@@ -2391,7 +2400,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="19" spans="1:6">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>42</v>
       </c>
@@ -2408,7 +2417,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>44</v>
       </c>
@@ -2425,7 +2434,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="21" spans="1:6">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>46</v>
       </c>
@@ -2442,7 +2451,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="22" spans="1:6">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>47</v>
       </c>
@@ -2459,7 +2468,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>49</v>
       </c>
@@ -2476,7 +2485,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="24" spans="1:6">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>52</v>
       </c>
@@ -2490,7 +2499,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="25" spans="1:6">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>53</v>
       </c>
@@ -2507,7 +2516,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="26" spans="1:6">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>56</v>
       </c>
@@ -2524,7 +2533,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="27" spans="1:6">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>58</v>
       </c>
@@ -2538,7 +2547,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="28" spans="1:6">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>59</v>
       </c>
@@ -2555,7 +2564,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="29" spans="1:6">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>61</v>
       </c>
@@ -2569,7 +2578,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="30" spans="1:6">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>63</v>
       </c>
@@ -2586,7 +2595,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>64</v>
       </c>
@@ -2603,7 +2612,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>67</v>
       </c>
@@ -2617,7 +2626,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="33" spans="1:6">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>68</v>
       </c>
@@ -2634,7 +2643,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="34" spans="1:6">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>69</v>
       </c>
@@ -2651,7 +2660,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="35" spans="1:6">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>72</v>
       </c>
@@ -2665,7 +2674,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="36" spans="1:6">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>73</v>
       </c>
@@ -2679,7 +2688,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="37" spans="1:6">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>74</v>
       </c>
@@ -2696,7 +2705,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="38" spans="1:6">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>77</v>
       </c>
@@ -2713,7 +2722,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="39" spans="1:6">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>78</v>
       </c>
@@ -2727,7 +2736,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="40" spans="1:6">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>80</v>
       </c>
@@ -2744,7 +2753,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="41" spans="1:6">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>82</v>
       </c>
@@ -2761,7 +2770,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="42" spans="1:6">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>84</v>
       </c>
@@ -2778,7 +2787,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="43" spans="1:6">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>86</v>
       </c>
@@ -2795,7 +2804,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="44" spans="1:6">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>90</v>
       </c>
@@ -2809,7 +2818,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="45" spans="1:6">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>91</v>
       </c>
@@ -2823,7 +2832,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="46" spans="1:6">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>92</v>
       </c>
@@ -2837,7 +2846,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="47" spans="1:6">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>93</v>
       </c>
@@ -2851,7 +2860,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="48" spans="1:6">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>94</v>
       </c>
@@ -2865,7 +2874,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="49" spans="1:6">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>95</v>
       </c>
@@ -2882,7 +2891,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="50" spans="1:6">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>97</v>
       </c>
@@ -2899,7 +2908,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="51" spans="1:6">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>98</v>
       </c>
@@ -2913,7 +2922,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="52" spans="1:6">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>100</v>
       </c>
@@ -2930,7 +2939,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="53" spans="1:6">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>103</v>
       </c>
@@ -2944,7 +2953,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="54" spans="1:6">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>104</v>
       </c>
@@ -2958,7 +2967,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="55" spans="1:6">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>105</v>
       </c>
@@ -2972,7 +2981,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="56" spans="1:6">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>106</v>
       </c>
@@ -2989,7 +2998,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="57" spans="1:6">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>108</v>
       </c>
@@ -3003,7 +3012,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="58" spans="1:6">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>110</v>
       </c>
@@ -3020,7 +3029,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="59" spans="1:6">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>112</v>
       </c>
@@ -3037,7 +3046,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="60" spans="1:6">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>113</v>
       </c>
@@ -3054,7 +3063,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="61" spans="1:6">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>115</v>
       </c>
@@ -3068,7 +3077,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="62" spans="1:6">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>116</v>
       </c>
@@ -3079,7 +3088,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="63" spans="1:6">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>117</v>
       </c>
@@ -3090,7 +3099,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="64" spans="1:6">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>118</v>
       </c>
@@ -3107,7 +3116,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="65" spans="1:6">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>120</v>
       </c>
@@ -3124,7 +3133,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="66" spans="1:6">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>122</v>
       </c>
@@ -3138,7 +3147,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="67" spans="1:6">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>123</v>
       </c>
@@ -3152,7 +3161,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="68" spans="1:6">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>124</v>
       </c>
@@ -3166,7 +3175,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="69" spans="1:6">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>125</v>
       </c>
@@ -3183,7 +3192,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="70" spans="1:6">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>128</v>
       </c>
@@ -3197,7 +3206,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="71" spans="1:6">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>129</v>
       </c>
@@ -3211,7 +3220,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="72" spans="1:6">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>130</v>
       </c>
@@ -3228,7 +3237,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="73" spans="1:6">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>132</v>
       </c>
@@ -3242,7 +3251,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="74" spans="1:6">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>134</v>
       </c>
@@ -3256,7 +3265,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="75" spans="1:6">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>136</v>
       </c>
@@ -3270,7 +3279,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="76" spans="1:6">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>137</v>
       </c>
@@ -3284,7 +3293,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="77" spans="1:6">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>138</v>
       </c>
@@ -3298,7 +3307,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="78" spans="1:6">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>139</v>
       </c>
@@ -3312,7 +3321,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="79" spans="1:6">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>140</v>
       </c>
@@ -3329,7 +3338,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="80" spans="1:6">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>142</v>
       </c>
@@ -3343,7 +3352,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="81" spans="1:6">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>143</v>
       </c>
@@ -3357,7 +3366,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="82" spans="1:6">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>144</v>
       </c>
@@ -3374,7 +3383,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="83" spans="1:6">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>146</v>
       </c>
@@ -3391,7 +3400,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="84" spans="1:6">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>149</v>
       </c>
@@ -3408,7 +3417,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="85" spans="1:6">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>151</v>
       </c>
@@ -3425,7 +3434,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="86" spans="1:6">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>152</v>
       </c>
@@ -3442,7 +3451,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="87" spans="1:6">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>154</v>
       </c>
@@ -3456,7 +3465,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="88" spans="1:6">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>155</v>
       </c>
@@ -3470,7 +3479,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="89" spans="1:6">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>157</v>
       </c>
@@ -3484,7 +3493,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="90" spans="1:6">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>158</v>
       </c>
@@ -3501,7 +3510,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="91" spans="1:6">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>159</v>
       </c>
@@ -3518,7 +3527,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="92" spans="1:6">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>161</v>
       </c>
@@ -3535,7 +3544,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="93" spans="1:6">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>163</v>
       </c>
@@ -3549,7 +3558,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="94" spans="1:6">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>164</v>
       </c>
@@ -3566,7 +3575,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="95" spans="1:6">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>166</v>
       </c>
@@ -3583,7 +3592,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="96" spans="1:6">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>168</v>
       </c>
@@ -3597,7 +3606,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="97" spans="1:6">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>169</v>
       </c>
@@ -3614,7 +3623,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="98" spans="1:6">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>171</v>
       </c>
@@ -3628,7 +3637,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="99" spans="1:6">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>172</v>
       </c>
@@ -3645,7 +3654,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="100" spans="1:6">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>174</v>
       </c>
@@ -3659,7 +3668,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="101" spans="1:6">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>175</v>
       </c>
@@ -3676,7 +3685,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="102" spans="1:6">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>176</v>
       </c>
@@ -3693,7 +3702,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="103" spans="1:6">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>178</v>
       </c>
@@ -3704,7 +3713,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="104" spans="1:6">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>179</v>
       </c>
@@ -3721,7 +3730,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="105" spans="1:6">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>181</v>
       </c>
@@ -3738,7 +3747,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="106" spans="1:6">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>183</v>
       </c>
@@ -3752,7 +3761,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="107" spans="1:6">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>184</v>
       </c>
@@ -3769,7 +3778,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="108" spans="1:6">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>185</v>
       </c>
@@ -3786,7 +3795,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="109" spans="1:6">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>187</v>
       </c>
@@ -3800,7 +3809,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="110" spans="1:6">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>188</v>
       </c>
@@ -3814,7 +3823,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="111" spans="1:6">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>189</v>
       </c>
@@ -3831,7 +3840,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="112" spans="1:6">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>191</v>
       </c>
@@ -3845,7 +3854,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="113" spans="1:6">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>192</v>
       </c>
@@ -3859,7 +3868,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="114" spans="1:6">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>193</v>
       </c>
@@ -3876,7 +3885,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="115" spans="1:6">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>195</v>
       </c>
@@ -3893,7 +3902,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="116" spans="1:6">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>197</v>
       </c>
@@ -3907,7 +3916,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="117" spans="1:6">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>199</v>
       </c>
@@ -3921,7 +3930,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="118" spans="1:6">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>201</v>
       </c>
@@ -3938,7 +3947,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="119" spans="1:6">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>204</v>
       </c>
@@ -3955,7 +3964,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="120" spans="1:6">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>205</v>
       </c>
@@ -3972,7 +3981,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="121" spans="1:6">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>207</v>
       </c>
@@ -3986,7 +3995,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="122" spans="1:6">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>208</v>
       </c>
@@ -4003,7 +4012,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="123" spans="1:6">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>210</v>
       </c>
@@ -4020,7 +4029,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="124" spans="1:6">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>211</v>
       </c>
@@ -4037,7 +4046,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="125" spans="1:6">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>212</v>
       </c>
@@ -4054,7 +4063,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="126" spans="1:6">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>213</v>
       </c>
@@ -4071,7 +4080,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="127" spans="1:6">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>214</v>
       </c>
@@ -4085,7 +4094,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="128" spans="1:6">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>215</v>
       </c>
@@ -4099,7 +4108,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="129" spans="1:6">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>216</v>
       </c>
@@ -4113,7 +4122,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="130" spans="1:6">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>217</v>
       </c>
@@ -4127,7 +4136,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="131" spans="1:6">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>218</v>
       </c>
@@ -4144,7 +4153,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="132" spans="1:6">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>220</v>
       </c>
@@ -4161,7 +4170,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="133" spans="1:6">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>222</v>
       </c>
@@ -4175,7 +4184,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="134" spans="1:6">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>223</v>
       </c>
@@ -4192,7 +4201,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="135" spans="1:6">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>224</v>
       </c>
@@ -4206,7 +4215,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="136" spans="1:6">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>225</v>
       </c>
@@ -4220,7 +4229,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="137" spans="1:6">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>226</v>
       </c>
@@ -4234,7 +4243,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="138" spans="1:6">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>227</v>
       </c>
@@ -4248,7 +4257,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="139" spans="1:6">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>228</v>
       </c>
@@ -4265,7 +4274,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="140" spans="1:6">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>230</v>
       </c>
@@ -4279,7 +4288,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="141" spans="1:6">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>231</v>
       </c>
@@ -4293,7 +4302,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="142" spans="1:6">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>233</v>
       </c>
@@ -4307,7 +4316,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="143" spans="1:6">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>235</v>
       </c>
@@ -4321,7 +4330,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="144" spans="1:6">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>237</v>
       </c>
@@ -4335,7 +4344,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="145" spans="1:6">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>239</v>
       </c>
@@ -4349,7 +4358,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="146" spans="1:6">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>241</v>
       </c>
@@ -4363,7 +4372,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="147" spans="1:6">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>243</v>
       </c>
@@ -4377,7 +4386,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="148" spans="1:6">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>245</v>
       </c>
@@ -4391,7 +4400,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="149" spans="1:6">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>247</v>
       </c>
@@ -4405,7 +4414,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="150" spans="1:6">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>248</v>
       </c>
@@ -4422,7 +4431,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="151" spans="1:6">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>251</v>
       </c>
@@ -4436,7 +4445,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="152" spans="1:6">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>253</v>
       </c>
@@ -4450,7 +4459,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="153" spans="1:6">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>254</v>
       </c>
@@ -4467,7 +4476,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="154" spans="1:6">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>256</v>
       </c>
@@ -4484,7 +4493,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="155" spans="1:6">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>258</v>
       </c>
@@ -4501,7 +4510,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="156" spans="1:6">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>260</v>
       </c>
@@ -4518,7 +4527,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="157" spans="1:6">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>261</v>
       </c>
@@ -4535,7 +4544,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="158" spans="1:6">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>263</v>
       </c>
@@ -4549,7 +4558,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="159" spans="1:6">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>264</v>
       </c>
@@ -4566,7 +4575,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="160" spans="1:6">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
         <v>265</v>
       </c>
@@ -4583,7 +4592,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="161" spans="1:6">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
         <v>267</v>
       </c>
@@ -4600,7 +4609,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="162" spans="1:6">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
         <v>268</v>
       </c>
@@ -4617,7 +4626,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="163" spans="1:6">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
         <v>271</v>
       </c>
@@ -4634,7 +4643,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="164" spans="1:6">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
         <v>273</v>
       </c>
@@ -4648,7 +4657,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="165" spans="1:6">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
         <v>274</v>
       </c>
@@ -4665,7 +4674,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="166" spans="1:6">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
         <v>275</v>
       </c>
@@ -4682,7 +4691,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="167" spans="1:6">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
         <v>277</v>
       </c>
@@ -4699,7 +4708,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="168" spans="1:6">
+    <row r="168" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
         <v>279</v>
       </c>
@@ -4716,7 +4725,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="169" spans="1:6">
+    <row r="169" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
         <v>281</v>
       </c>
@@ -4733,7 +4742,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="170" spans="1:6">
+    <row r="170" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
         <v>283</v>
       </c>
@@ -4750,7 +4759,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="171" spans="1:6">
+    <row r="171" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
         <v>286</v>
       </c>
@@ -4767,7 +4776,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="172" spans="1:6">
+    <row r="172" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
         <v>288</v>
       </c>
@@ -4784,7 +4793,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="173" spans="1:6">
+    <row r="173" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
         <v>290</v>
       </c>
@@ -4798,7 +4807,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="174" spans="1:6">
+    <row r="174" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
         <v>292</v>
       </c>
@@ -4812,7 +4821,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="175" spans="1:6">
+    <row r="175" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
         <v>294</v>
       </c>
@@ -4829,7 +4838,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="176" spans="1:6">
+    <row r="176" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
         <v>297</v>
       </c>
@@ -4846,7 +4855,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="177" spans="1:6">
+    <row r="177" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>300</v>
       </c>
@@ -4863,7 +4872,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="178" spans="1:6">
+    <row r="178" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>301</v>
       </c>
@@ -4880,7 +4889,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="179" spans="1:6">
+    <row r="179" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>303</v>
       </c>
@@ -4897,7 +4906,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="180" spans="1:6">
+    <row r="180" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
         <v>305</v>
       </c>
@@ -4914,7 +4923,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="181" spans="1:6">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
         <v>307</v>
       </c>
@@ -4931,7 +4940,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="182" spans="1:6">
+    <row r="182" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
         <v>309</v>
       </c>
@@ -4948,7 +4957,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="183" spans="1:6">
+    <row r="183" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
         <v>310</v>
       </c>
@@ -4962,7 +4971,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="184" spans="1:6">
+    <row r="184" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
         <v>311</v>
       </c>
@@ -4979,7 +4988,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="185" spans="1:6">
+    <row r="185" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
         <v>313</v>
       </c>
@@ -4996,7 +5005,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="186" spans="1:6">
+    <row r="186" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
         <v>314</v>
       </c>
@@ -5013,7 +5022,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="187" spans="1:6">
+    <row r="187" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
         <v>316</v>
       </c>
@@ -5027,7 +5036,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="188" spans="1:6">
+    <row r="188" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
         <v>317</v>
       </c>
@@ -5044,7 +5053,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="189" spans="1:6">
+    <row r="189" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
         <v>319</v>
       </c>
@@ -5061,7 +5070,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="190" spans="1:6">
+    <row r="190" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
         <v>320</v>
       </c>
@@ -5078,7 +5087,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="191" spans="1:6">
+    <row r="191" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
         <v>321</v>
       </c>
@@ -5095,7 +5104,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="192" spans="1:6">
+    <row r="192" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
         <v>323</v>
       </c>
@@ -5112,7 +5121,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="193" spans="1:6">
+    <row r="193" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
         <v>325</v>
       </c>
@@ -5129,7 +5138,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="194" spans="1:6">
+    <row r="194" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
         <v>327</v>
       </c>
@@ -5146,7 +5155,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="195" spans="1:6">
+    <row r="195" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
         <v>329</v>
       </c>
@@ -5160,7 +5169,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="196" spans="1:6">
+    <row r="196" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
         <v>331</v>
       </c>
@@ -5174,7 +5183,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="197" spans="1:6">
+    <row r="197" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
         <v>333</v>
       </c>
@@ -5191,7 +5200,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="198" spans="1:6">
+    <row r="198" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
         <v>335</v>
       </c>
@@ -5208,7 +5217,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="199" spans="1:6">
+    <row r="199" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
         <v>337</v>
       </c>
@@ -5222,7 +5231,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="200" spans="1:6">
+    <row r="200" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
         <v>339</v>
       </c>
@@ -5239,7 +5248,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="201" spans="1:6">
+    <row r="201" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
         <v>341</v>
       </c>
@@ -5253,7 +5262,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="202" spans="1:6">
+    <row r="202" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
         <v>343</v>
       </c>
@@ -5270,7 +5279,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="203" spans="1:6">
+    <row r="203" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
         <v>345</v>
       </c>
@@ -5287,7 +5296,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="204" spans="1:6">
+    <row r="204" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
         <v>347</v>
       </c>
@@ -5304,7 +5313,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="205" spans="1:6">
+    <row r="205" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
         <v>348</v>
       </c>
@@ -5318,7 +5327,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="206" spans="1:6">
+    <row r="206" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
         <v>349</v>
       </c>
@@ -5332,7 +5341,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="207" spans="1:6">
+    <row r="207" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
         <v>350</v>
       </c>
@@ -5349,7 +5358,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="208" spans="1:6">
+    <row r="208" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
         <v>352</v>
       </c>
@@ -5366,7 +5375,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="209" spans="1:6">
+    <row r="209" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
         <v>354</v>
       </c>
@@ -5383,7 +5392,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="210" spans="1:6">
+    <row r="210" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
         <v>356</v>
       </c>
@@ -5400,7 +5409,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="211" spans="1:6">
+    <row r="211" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
         <v>358</v>
       </c>
@@ -5417,7 +5426,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="212" spans="1:6">
+    <row r="212" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
         <v>359</v>
       </c>
@@ -5431,7 +5440,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="213" spans="1:6">
+    <row r="213" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
         <v>360</v>
       </c>
@@ -5448,7 +5457,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="214" spans="1:6">
+    <row r="214" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
         <v>362</v>
       </c>
@@ -5462,7 +5471,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="215" spans="1:6">
+    <row r="215" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A215" t="s">
         <v>363</v>
       </c>
@@ -5476,7 +5485,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="216" spans="1:6">
+    <row r="216" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A216" t="s">
         <v>365</v>
       </c>
@@ -5490,7 +5499,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="217" spans="1:6">
+    <row r="217" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
         <v>367</v>
       </c>
@@ -5507,7 +5516,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="218" spans="1:6">
+    <row r="218" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A218" t="s">
         <v>369</v>
       </c>
@@ -5524,7 +5533,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="219" spans="1:6">
+    <row r="219" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
         <v>371</v>
       </c>
@@ -5538,7 +5547,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="220" spans="1:6">
+    <row r="220" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
         <v>372</v>
       </c>
@@ -5555,7 +5564,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="221" spans="1:6">
+    <row r="221" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
         <v>374</v>
       </c>
@@ -5572,7 +5581,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="222" spans="1:6">
+    <row r="222" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
         <v>375</v>
       </c>
@@ -5586,7 +5595,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="223" spans="1:6">
+    <row r="223" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
         <v>376</v>
       </c>
@@ -5603,7 +5612,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="224" spans="1:6">
+    <row r="224" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
         <v>377</v>
       </c>
@@ -5620,7 +5629,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="225" spans="1:6">
+    <row r="225" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
         <v>379</v>
       </c>
@@ -5637,7 +5646,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="226" spans="1:6">
+    <row r="226" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
         <v>381</v>
       </c>
@@ -5654,7 +5663,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="227" spans="1:6">
+    <row r="227" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
         <v>383</v>
       </c>
@@ -5668,7 +5677,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="228" spans="1:6">
+    <row r="228" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A228" t="s">
         <v>384</v>
       </c>
@@ -5682,7 +5691,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="229" spans="1:6">
+    <row r="229" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
         <v>386</v>
       </c>
@@ -5699,7 +5708,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="230" spans="1:6">
+    <row r="230" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
         <v>388</v>
       </c>
@@ -5716,7 +5725,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="231" spans="1:6">
+    <row r="231" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A231" t="s">
         <v>390</v>
       </c>
@@ -5730,7 +5739,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="232" spans="1:6">
+    <row r="232" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A232" t="s">
         <v>391</v>
       </c>
@@ -5744,7 +5753,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="233" spans="1:6">
+    <row r="233" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
         <v>393</v>
       </c>
@@ -5761,7 +5770,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="234" spans="1:6">
+    <row r="234" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
         <v>395</v>
       </c>
@@ -5778,7 +5787,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="235" spans="1:6">
+    <row r="235" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A235" t="s">
         <v>397</v>
       </c>
@@ -5795,7 +5804,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="236" spans="1:6">
+    <row r="236" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
         <v>399</v>
       </c>
@@ -5812,7 +5821,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="237" spans="1:6">
+    <row r="237" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
         <v>401</v>
       </c>
@@ -5829,7 +5838,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="238" spans="1:6">
+    <row r="238" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
         <v>403</v>
       </c>
@@ -5846,7 +5855,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="239" spans="1:6">
+    <row r="239" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A239" t="s">
         <v>405</v>
       </c>
@@ -5860,7 +5869,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="240" spans="1:6">
+    <row r="240" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A240" t="s">
         <v>407</v>
       </c>
@@ -5874,7 +5883,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="241" spans="1:6">
+    <row r="241" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
         <v>409</v>
       </c>
@@ -5891,7 +5900,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="242" spans="1:6">
+    <row r="242" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
         <v>410</v>
       </c>
@@ -5905,7 +5914,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="243" spans="1:6">
+    <row r="243" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A243" t="s">
         <v>411</v>
       </c>
@@ -5919,7 +5928,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="244" spans="1:6">
+    <row r="244" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A244" t="s">
         <v>412</v>
       </c>
@@ -5936,7 +5945,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="245" spans="1:6">
+    <row r="245" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A245" t="s">
         <v>413</v>
       </c>
@@ -5953,7 +5962,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="246" spans="1:6">
+    <row r="246" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A246" t="s">
         <v>414</v>
       </c>
@@ -5970,7 +5979,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="247" spans="1:6">
+    <row r="247" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A247" t="s">
         <v>415</v>
       </c>
@@ -5987,7 +5996,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="248" spans="1:6">
+    <row r="248" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A248" t="s">
         <v>418</v>
       </c>
@@ -6004,7 +6013,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="249" spans="1:6">
+    <row r="249" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A249" t="s">
         <v>419</v>
       </c>
@@ -6018,7 +6027,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="250" spans="1:6">
+    <row r="250" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
         <v>420</v>
       </c>
@@ -6032,7 +6041,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="251" spans="1:6">
+    <row r="251" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A251" t="s">
         <v>421</v>
       </c>
@@ -6046,7 +6055,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="252" spans="1:6">
+    <row r="252" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A252" t="s">
         <v>422</v>
       </c>
@@ -6063,7 +6072,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="253" spans="1:6">
+    <row r="253" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A253" t="s">
         <v>424</v>
       </c>
@@ -6080,7 +6089,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="254" spans="1:6">
+    <row r="254" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A254" t="s">
         <v>426</v>
       </c>
@@ -6097,7 +6106,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="255" spans="1:6">
+    <row r="255" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A255" t="s">
         <v>428</v>
       </c>
@@ -6111,7 +6120,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="256" spans="1:6">
+    <row r="256" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A256" t="s">
         <v>429</v>
       </c>
@@ -6128,7 +6137,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="257" spans="1:6">
+    <row r="257" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A257" t="s">
         <v>430</v>
       </c>
@@ -6142,7 +6151,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="258" spans="1:6">
+    <row r="258" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A258" t="s">
         <v>431</v>
       </c>
@@ -6156,7 +6165,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="259" spans="1:6">
+    <row r="259" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A259" t="s">
         <v>432</v>
       </c>
@@ -6173,7 +6182,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="260" spans="1:6">
+    <row r="260" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A260" t="s">
         <v>434</v>
       </c>
@@ -6190,7 +6199,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="261" spans="1:6">
+    <row r="261" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A261" t="s">
         <v>435</v>
       </c>
@@ -6207,7 +6216,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="262" spans="1:6">
+    <row r="262" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A262" t="s">
         <v>437</v>
       </c>
@@ -6221,7 +6230,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="263" spans="1:6">
+    <row r="263" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A263" t="s">
         <v>439</v>
       </c>
@@ -6235,7 +6244,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="264" spans="1:6">
+    <row r="264" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A264" t="s">
         <v>441</v>
       </c>
@@ -6249,7 +6258,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="265" spans="1:6">
+    <row r="265" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A265" t="s">
         <v>443</v>
       </c>
@@ -6263,7 +6272,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="266" spans="1:6">
+    <row r="266" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A266" t="s">
         <v>444</v>
       </c>
@@ -6277,7 +6286,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="267" spans="1:6">
+    <row r="267" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A267" t="s">
         <v>445</v>
       </c>
@@ -6291,7 +6300,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="268" spans="1:6">
+    <row r="268" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A268" t="s">
         <v>446</v>
       </c>
@@ -6305,7 +6314,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="269" spans="1:6">
+    <row r="269" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A269" t="s">
         <v>447</v>
       </c>
@@ -6319,7 +6328,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="270" spans="1:6">
+    <row r="270" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A270" t="s">
         <v>448</v>
       </c>
@@ -6336,7 +6345,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="271" spans="1:6">
+    <row r="271" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A271" t="s">
         <v>450</v>
       </c>
@@ -6353,7 +6362,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="272" spans="1:6">
+    <row r="272" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A272" t="s">
         <v>452</v>
       </c>
@@ -6367,7 +6376,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="273" spans="1:6">
+    <row r="273" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A273" t="s">
         <v>453</v>
       </c>
@@ -6384,7 +6393,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="274" spans="1:6">
+    <row r="274" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A274" t="s">
         <v>455</v>
       </c>
@@ -6398,7 +6407,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="275" spans="1:6">
+    <row r="275" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A275" t="s">
         <v>456</v>
       </c>
@@ -6412,7 +6421,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="276" spans="1:6">
+    <row r="276" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A276" t="s">
         <v>458</v>
       </c>
@@ -6426,7 +6435,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="277" spans="1:6">
+    <row r="277" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A277" t="s">
         <v>460</v>
       </c>
@@ -6440,7 +6449,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="278" spans="1:6">
+    <row r="278" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A278" t="s">
         <v>462</v>
       </c>
@@ -6454,7 +6463,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="279" spans="1:6">
+    <row r="279" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A279" t="s">
         <v>463</v>
       </c>
@@ -6468,7 +6477,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="280" spans="1:6">
+    <row r="280" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A280" t="s">
         <v>464</v>
       </c>
@@ -6485,7 +6494,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="281" spans="1:6">
+    <row r="281" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A281" t="s">
         <v>466</v>
       </c>
@@ -6502,7 +6511,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="282" spans="1:6">
+    <row r="282" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A282" t="s">
         <v>467</v>
       </c>
@@ -6516,7 +6525,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="283" spans="1:6">
+    <row r="283" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A283" t="s">
         <v>468</v>
       </c>
@@ -6533,7 +6542,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="284" spans="1:6">
+    <row r="284" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A284" t="s">
         <v>469</v>
       </c>
@@ -6550,7 +6559,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="285" spans="1:6">
+    <row r="285" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A285" t="s">
         <v>470</v>
       </c>
@@ -6567,7 +6576,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="286" spans="1:6">
+    <row r="286" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A286" t="s">
         <v>472</v>
       </c>
@@ -6584,7 +6593,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="287" spans="1:6">
+    <row r="287" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A287" t="s">
         <v>474</v>
       </c>
@@ -6601,7 +6610,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="288" spans="1:6">
+    <row r="288" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A288" t="s">
         <v>475</v>
       </c>
@@ -6618,7 +6627,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="289" spans="1:6">
+    <row r="289" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A289" t="s">
         <v>477</v>
       </c>
@@ -6635,7 +6644,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="290" spans="1:6">
+    <row r="290" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A290" t="s">
         <v>478</v>
       </c>
@@ -6652,7 +6661,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="291" spans="1:6">
+    <row r="291" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A291" t="s">
         <v>479</v>
       </c>
@@ -6669,7 +6678,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="292" spans="1:6">
+    <row r="292" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A292" t="s">
         <v>480</v>
       </c>
@@ -6686,7 +6695,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="293" spans="1:6">
+    <row r="293" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A293" t="s">
         <v>482</v>
       </c>
@@ -6703,7 +6712,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="294" spans="1:6">
+    <row r="294" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A294" t="s">
         <v>484</v>
       </c>
@@ -6720,7 +6729,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="295" spans="1:6">
+    <row r="295" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A295" t="s">
         <v>486</v>
       </c>
@@ -6737,7 +6746,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="296" spans="1:6">
+    <row r="296" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A296" t="s">
         <v>488</v>
       </c>
@@ -6754,7 +6763,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="297" spans="1:6">
+    <row r="297" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A297" t="s">
         <v>489</v>
       </c>
@@ -6771,7 +6780,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="298" spans="1:6">
+    <row r="298" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A298" t="s">
         <v>491</v>
       </c>
@@ -6788,7 +6797,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="299" spans="1:6">
+    <row r="299" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A299" t="s">
         <v>492</v>
       </c>
@@ -6805,7 +6814,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="300" spans="1:6">
+    <row r="300" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A300" t="s">
         <v>550</v>
       </c>
@@ -6816,7 +6825,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="301" spans="1:6">
+    <row r="301" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A301" t="s">
         <v>549</v>
       </c>
@@ -6827,7 +6836,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="302" spans="1:6">
+    <row r="302" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A302" t="s">
         <v>548</v>
       </c>
@@ -6838,18 +6847,18 @@
         <v>493</v>
       </c>
     </row>
-    <row r="303" spans="1:6">
+    <row r="303" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A303" t="s">
         <v>547</v>
       </c>
       <c r="C303" t="s">
-        <v>551</v>
+        <v>552</v>
       </c>
       <c r="F303" t="s">
         <v>493</v>
       </c>
     </row>
-    <row r="304" spans="1:6">
+    <row r="304" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A304" t="s">
         <v>546</v>
       </c>
@@ -6860,7 +6869,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="305" spans="1:6">
+    <row r="305" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A305" t="s">
         <v>545</v>
       </c>
@@ -6871,7 +6880,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="306" spans="1:6">
+    <row r="306" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A306" t="s">
         <v>544</v>
       </c>
@@ -6879,6 +6888,20 @@
         <v>543</v>
       </c>
       <c r="F306" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="307" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A307" t="s">
+        <v>551</v>
+      </c>
+      <c r="C307" t="s">
+        <v>553</v>
+      </c>
+      <c r="E307" t="s">
+        <v>554</v>
+      </c>
+      <c r="F307" t="s">
         <v>493</v>
       </c>
     </row>
@@ -6891,9 +6914,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E009BBAC-B988-7C49-8FAA-EA75972BA821}">
   <dimension ref="A1:B18"/>
-  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>146</v>
       </c>
@@ -6901,7 +6924,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="2" spans="1:2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>155</v>
       </c>
@@ -6909,7 +6932,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>100</v>
       </c>
@@ -6917,7 +6940,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>98</v>
       </c>
@@ -6925,7 +6948,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>248</v>
       </c>
@@ -6933,7 +6956,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>251</v>
       </c>
@@ -6941,7 +6964,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>176</v>
       </c>
@@ -6949,7 +6972,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="8" spans="1:2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>199</v>
       </c>
@@ -6957,7 +6980,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>239</v>
       </c>
@@ -6965,7 +6988,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>245</v>
       </c>
@@ -6973,7 +6996,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" s="2" t="s">
         <v>235</v>
       </c>
@@ -6981,7 +7004,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="12" spans="1:2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>237</v>
       </c>
@@ -6989,7 +7012,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="13" spans="1:2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>241</v>
       </c>
@@ -6997,7 +7020,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="14" spans="1:2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>243</v>
       </c>
@@ -7005,7 +7028,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="15" spans="1:2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>231</v>
       </c>
@@ -7013,7 +7036,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="16" spans="1:2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>233</v>
       </c>
@@ -7021,7 +7044,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="17" spans="1:2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>500</v>
       </c>
@@ -7029,7 +7052,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="18" spans="1:2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>502</v>
       </c>

</xml_diff>

<commit_message>
Remove unnecessary whitespace in pipeline-content.json
</commit_message>
<xml_diff>
--- a/documentation/workflow/bc_bronze_workflow_mapping.xlsx
+++ b/documentation/workflow/bc_bronze_workflow_mapping.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fantasysuperkick/workspace/ccg/datawarehouse/documentation/workflow/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Documents\Exco_Partners\Data-Warehouse\documentation\workflow\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{910E5B33-68BC-0747-B38C-2D1A38332D93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F21415FF-7DCC-4CBA-90CC-6C8543EAC77A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="660" yWindow="500" windowWidth="23260" windowHeight="12460" xr2:uid="{2F7A961D-90EA-0F4A-9BBB-FA6BCAC4A400}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{2F7A961D-90EA-0F4A-9BBB-FA6BCAC4A400}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1698,20 +1698,20 @@
     <t>DimensionSetEntry</t>
   </si>
   <si>
-    <t>sourcetype, sourcessubtype, sourceno,  locationcode, type, company, source_system</t>
-  </si>
-  <si>
     <t>dimensionsetid, dimensioncode,company, source_system</t>
   </si>
   <si>
     <t>dimensionvaluecode,globaldimensionno</t>
+  </si>
+  <si>
+    <t>sourcetype, sourcesubtype, sourceno,  locationcode, type, company, source_system</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="3">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -2100,16 +2100,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E95DFF8-97A2-F246-A8EF-BFAEB7CC069C}">
   <dimension ref="A1:F307"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6"/>
   <cols>
-    <col min="1" max="2" width="22.1640625" customWidth="1"/>
-    <col min="3" max="3" width="72.1640625" customWidth="1"/>
-    <col min="4" max="4" width="59.6640625" customWidth="1"/>
-    <col min="5" max="5" width="49.83203125" customWidth="1"/>
-    <col min="6" max="6" width="20.6640625" customWidth="1"/>
+    <col min="1" max="2" width="22.19921875" customWidth="1"/>
+    <col min="3" max="3" width="72.19921875" customWidth="1"/>
+    <col min="4" max="4" width="59.69921875" customWidth="1"/>
+    <col min="5" max="5" width="49.796875" customWidth="1"/>
+    <col min="6" max="6" width="20.69921875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
         <v>504</v>
       </c>
@@ -2129,7 +2129,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2146,7 +2146,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2163,7 +2163,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -2177,7 +2177,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2191,7 +2191,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -2208,7 +2208,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -2222,7 +2222,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -2239,7 +2239,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -2253,7 +2253,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -2270,7 +2270,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -2287,7 +2287,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -2304,7 +2304,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6">
       <c r="A13" t="s">
         <v>26</v>
       </c>
@@ -2321,7 +2321,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6">
       <c r="A14" t="s">
         <v>28</v>
       </c>
@@ -2338,7 +2338,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -2355,7 +2355,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6">
       <c r="A16" t="s">
         <v>35</v>
       </c>
@@ -2369,7 +2369,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6">
       <c r="A17" t="s">
         <v>36</v>
       </c>
@@ -2386,7 +2386,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6">
       <c r="A18" t="s">
         <v>39</v>
       </c>
@@ -2400,7 +2400,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6">
       <c r="A19" t="s">
         <v>42</v>
       </c>
@@ -2417,7 +2417,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6">
       <c r="A20" t="s">
         <v>44</v>
       </c>
@@ -2434,7 +2434,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6">
       <c r="A21" t="s">
         <v>46</v>
       </c>
@@ -2451,7 +2451,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6">
       <c r="A22" t="s">
         <v>47</v>
       </c>
@@ -2468,7 +2468,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6">
       <c r="A23" t="s">
         <v>49</v>
       </c>
@@ -2485,7 +2485,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6">
       <c r="A24" t="s">
         <v>52</v>
       </c>
@@ -2499,7 +2499,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6">
       <c r="A25" t="s">
         <v>53</v>
       </c>
@@ -2516,7 +2516,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6">
       <c r="A26" t="s">
         <v>56</v>
       </c>
@@ -2533,7 +2533,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6">
       <c r="A27" t="s">
         <v>58</v>
       </c>
@@ -2547,7 +2547,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6">
       <c r="A28" t="s">
         <v>59</v>
       </c>
@@ -2564,7 +2564,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6">
       <c r="A29" t="s">
         <v>61</v>
       </c>
@@ -2578,7 +2578,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6">
       <c r="A30" t="s">
         <v>63</v>
       </c>
@@ -2595,7 +2595,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6">
       <c r="A31" t="s">
         <v>64</v>
       </c>
@@ -2612,7 +2612,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6">
       <c r="A32" t="s">
         <v>67</v>
       </c>
@@ -2626,7 +2626,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6">
       <c r="A33" t="s">
         <v>68</v>
       </c>
@@ -2643,7 +2643,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6">
       <c r="A34" t="s">
         <v>69</v>
       </c>
@@ -2660,7 +2660,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6">
       <c r="A35" t="s">
         <v>72</v>
       </c>
@@ -2674,7 +2674,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6">
       <c r="A36" t="s">
         <v>73</v>
       </c>
@@ -2688,7 +2688,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6">
       <c r="A37" t="s">
         <v>74</v>
       </c>
@@ -2705,7 +2705,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6">
       <c r="A38" t="s">
         <v>77</v>
       </c>
@@ -2722,7 +2722,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6">
       <c r="A39" t="s">
         <v>78</v>
       </c>
@@ -2736,7 +2736,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6">
       <c r="A40" t="s">
         <v>80</v>
       </c>
@@ -2753,7 +2753,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6">
       <c r="A41" t="s">
         <v>82</v>
       </c>
@@ -2770,7 +2770,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6">
       <c r="A42" t="s">
         <v>84</v>
       </c>
@@ -2787,7 +2787,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6">
       <c r="A43" t="s">
         <v>86</v>
       </c>
@@ -2804,7 +2804,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6">
       <c r="A44" t="s">
         <v>90</v>
       </c>
@@ -2818,7 +2818,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6">
       <c r="A45" t="s">
         <v>91</v>
       </c>
@@ -2832,7 +2832,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6">
       <c r="A46" t="s">
         <v>92</v>
       </c>
@@ -2846,7 +2846,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6">
       <c r="A47" t="s">
         <v>93</v>
       </c>
@@ -2860,7 +2860,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6">
       <c r="A48" t="s">
         <v>94</v>
       </c>
@@ -2874,7 +2874,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6">
       <c r="A49" t="s">
         <v>95</v>
       </c>
@@ -2891,7 +2891,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6">
       <c r="A50" t="s">
         <v>97</v>
       </c>
@@ -2908,7 +2908,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6">
       <c r="A51" t="s">
         <v>98</v>
       </c>
@@ -2922,7 +2922,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:6">
       <c r="A52" t="s">
         <v>100</v>
       </c>
@@ -2939,7 +2939,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:6">
       <c r="A53" t="s">
         <v>103</v>
       </c>
@@ -2953,7 +2953,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:6">
       <c r="A54" t="s">
         <v>104</v>
       </c>
@@ -2967,7 +2967,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:6">
       <c r="A55" t="s">
         <v>105</v>
       </c>
@@ -2981,7 +2981,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:6">
       <c r="A56" t="s">
         <v>106</v>
       </c>
@@ -2998,7 +2998,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:6">
       <c r="A57" t="s">
         <v>108</v>
       </c>
@@ -3012,7 +3012,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:6">
       <c r="A58" t="s">
         <v>110</v>
       </c>
@@ -3029,7 +3029,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:6">
       <c r="A59" t="s">
         <v>112</v>
       </c>
@@ -3046,7 +3046,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:6">
       <c r="A60" t="s">
         <v>113</v>
       </c>
@@ -3063,7 +3063,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:6">
       <c r="A61" t="s">
         <v>115</v>
       </c>
@@ -3077,7 +3077,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:6">
       <c r="A62" t="s">
         <v>116</v>
       </c>
@@ -3088,7 +3088,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:6">
       <c r="A63" t="s">
         <v>117</v>
       </c>
@@ -3099,7 +3099,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:6">
       <c r="A64" t="s">
         <v>118</v>
       </c>
@@ -3116,7 +3116,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:6">
       <c r="A65" t="s">
         <v>120</v>
       </c>
@@ -3133,7 +3133,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:6">
       <c r="A66" t="s">
         <v>122</v>
       </c>
@@ -3147,7 +3147,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:6">
       <c r="A67" t="s">
         <v>123</v>
       </c>
@@ -3161,7 +3161,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:6">
       <c r="A68" t="s">
         <v>124</v>
       </c>
@@ -3175,7 +3175,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:6">
       <c r="A69" t="s">
         <v>125</v>
       </c>
@@ -3192,7 +3192,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:6">
       <c r="A70" t="s">
         <v>128</v>
       </c>
@@ -3206,7 +3206,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:6">
       <c r="A71" t="s">
         <v>129</v>
       </c>
@@ -3220,7 +3220,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:6">
       <c r="A72" t="s">
         <v>130</v>
       </c>
@@ -3237,7 +3237,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:6">
       <c r="A73" t="s">
         <v>132</v>
       </c>
@@ -3251,7 +3251,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:6">
       <c r="A74" t="s">
         <v>134</v>
       </c>
@@ -3265,7 +3265,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:6">
       <c r="A75" t="s">
         <v>136</v>
       </c>
@@ -3279,7 +3279,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:6">
       <c r="A76" t="s">
         <v>137</v>
       </c>
@@ -3293,7 +3293,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:6">
       <c r="A77" t="s">
         <v>138</v>
       </c>
@@ -3307,7 +3307,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:6">
       <c r="A78" t="s">
         <v>139</v>
       </c>
@@ -3321,7 +3321,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:6">
       <c r="A79" t="s">
         <v>140</v>
       </c>
@@ -3338,7 +3338,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:6">
       <c r="A80" t="s">
         <v>142</v>
       </c>
@@ -3352,7 +3352,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:6">
       <c r="A81" t="s">
         <v>143</v>
       </c>
@@ -3366,7 +3366,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:6">
       <c r="A82" t="s">
         <v>144</v>
       </c>
@@ -3383,7 +3383,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:6">
       <c r="A83" t="s">
         <v>146</v>
       </c>
@@ -3400,7 +3400,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:6">
       <c r="A84" t="s">
         <v>149</v>
       </c>
@@ -3417,7 +3417,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:6">
       <c r="A85" t="s">
         <v>151</v>
       </c>
@@ -3434,7 +3434,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:6">
       <c r="A86" t="s">
         <v>152</v>
       </c>
@@ -3451,7 +3451,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:6">
       <c r="A87" t="s">
         <v>154</v>
       </c>
@@ -3465,7 +3465,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:6">
       <c r="A88" t="s">
         <v>155</v>
       </c>
@@ -3479,7 +3479,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:6">
       <c r="A89" t="s">
         <v>157</v>
       </c>
@@ -3493,7 +3493,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:6">
       <c r="A90" t="s">
         <v>158</v>
       </c>
@@ -3510,7 +3510,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:6">
       <c r="A91" t="s">
         <v>159</v>
       </c>
@@ -3527,7 +3527,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:6">
       <c r="A92" t="s">
         <v>161</v>
       </c>
@@ -3544,7 +3544,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:6">
       <c r="A93" t="s">
         <v>163</v>
       </c>
@@ -3558,7 +3558,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:6">
       <c r="A94" t="s">
         <v>164</v>
       </c>
@@ -3575,7 +3575,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:6">
       <c r="A95" t="s">
         <v>166</v>
       </c>
@@ -3592,7 +3592,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:6">
       <c r="A96" t="s">
         <v>168</v>
       </c>
@@ -3606,7 +3606,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:6">
       <c r="A97" t="s">
         <v>169</v>
       </c>
@@ -3623,7 +3623,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:6">
       <c r="A98" t="s">
         <v>171</v>
       </c>
@@ -3637,7 +3637,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:6">
       <c r="A99" t="s">
         <v>172</v>
       </c>
@@ -3654,7 +3654,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:6">
       <c r="A100" t="s">
         <v>174</v>
       </c>
@@ -3668,7 +3668,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:6">
       <c r="A101" t="s">
         <v>175</v>
       </c>
@@ -3685,7 +3685,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:6">
       <c r="A102" t="s">
         <v>176</v>
       </c>
@@ -3702,7 +3702,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:6">
       <c r="A103" t="s">
         <v>178</v>
       </c>
@@ -3713,7 +3713,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:6">
       <c r="A104" t="s">
         <v>179</v>
       </c>
@@ -3730,7 +3730,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:6">
       <c r="A105" t="s">
         <v>181</v>
       </c>
@@ -3747,7 +3747,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:6">
       <c r="A106" t="s">
         <v>183</v>
       </c>
@@ -3761,7 +3761,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:6">
       <c r="A107" t="s">
         <v>184</v>
       </c>
@@ -3778,7 +3778,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:6">
       <c r="A108" t="s">
         <v>185</v>
       </c>
@@ -3795,7 +3795,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:6">
       <c r="A109" t="s">
         <v>187</v>
       </c>
@@ -3809,7 +3809,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:6">
       <c r="A110" t="s">
         <v>188</v>
       </c>
@@ -3823,7 +3823,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:6">
       <c r="A111" t="s">
         <v>189</v>
       </c>
@@ -3840,7 +3840,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:6">
       <c r="A112" t="s">
         <v>191</v>
       </c>
@@ -3854,7 +3854,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:6">
       <c r="A113" t="s">
         <v>192</v>
       </c>
@@ -3868,7 +3868,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:6">
       <c r="A114" t="s">
         <v>193</v>
       </c>
@@ -3885,7 +3885,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:6">
       <c r="A115" t="s">
         <v>195</v>
       </c>
@@ -3902,7 +3902,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:6">
       <c r="A116" t="s">
         <v>197</v>
       </c>
@@ -3916,7 +3916,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:6">
       <c r="A117" t="s">
         <v>199</v>
       </c>
@@ -3930,7 +3930,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:6">
       <c r="A118" t="s">
         <v>201</v>
       </c>
@@ -3947,7 +3947,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:6">
       <c r="A119" t="s">
         <v>204</v>
       </c>
@@ -3964,7 +3964,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:6">
       <c r="A120" t="s">
         <v>205</v>
       </c>
@@ -3981,7 +3981,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:6">
       <c r="A121" t="s">
         <v>207</v>
       </c>
@@ -3995,7 +3995,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:6">
       <c r="A122" t="s">
         <v>208</v>
       </c>
@@ -4012,7 +4012,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:6">
       <c r="A123" t="s">
         <v>210</v>
       </c>
@@ -4029,7 +4029,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:6">
       <c r="A124" t="s">
         <v>211</v>
       </c>
@@ -4046,7 +4046,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:6">
       <c r="A125" t="s">
         <v>212</v>
       </c>
@@ -4063,7 +4063,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:6">
       <c r="A126" t="s">
         <v>213</v>
       </c>
@@ -4080,7 +4080,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:6">
       <c r="A127" t="s">
         <v>214</v>
       </c>
@@ -4094,7 +4094,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:6">
       <c r="A128" t="s">
         <v>215</v>
       </c>
@@ -4108,7 +4108,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:6">
       <c r="A129" t="s">
         <v>216</v>
       </c>
@@ -4122,7 +4122,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:6">
       <c r="A130" t="s">
         <v>217</v>
       </c>
@@ -4136,7 +4136,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:6">
       <c r="A131" t="s">
         <v>218</v>
       </c>
@@ -4153,7 +4153,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:6">
       <c r="A132" t="s">
         <v>220</v>
       </c>
@@ -4170,7 +4170,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:6">
       <c r="A133" t="s">
         <v>222</v>
       </c>
@@ -4184,7 +4184,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:6">
       <c r="A134" t="s">
         <v>223</v>
       </c>
@@ -4201,7 +4201,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:6">
       <c r="A135" t="s">
         <v>224</v>
       </c>
@@ -4215,7 +4215,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:6">
       <c r="A136" t="s">
         <v>225</v>
       </c>
@@ -4229,7 +4229,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:6">
       <c r="A137" t="s">
         <v>226</v>
       </c>
@@ -4243,7 +4243,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:6">
       <c r="A138" t="s">
         <v>227</v>
       </c>
@@ -4257,7 +4257,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:6">
       <c r="A139" t="s">
         <v>228</v>
       </c>
@@ -4274,7 +4274,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:6">
       <c r="A140" t="s">
         <v>230</v>
       </c>
@@ -4288,7 +4288,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:6">
       <c r="A141" t="s">
         <v>231</v>
       </c>
@@ -4302,7 +4302,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:6">
       <c r="A142" t="s">
         <v>233</v>
       </c>
@@ -4316,7 +4316,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:6">
       <c r="A143" t="s">
         <v>235</v>
       </c>
@@ -4330,7 +4330,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:6">
       <c r="A144" t="s">
         <v>237</v>
       </c>
@@ -4344,7 +4344,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:6">
       <c r="A145" t="s">
         <v>239</v>
       </c>
@@ -4358,7 +4358,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:6">
       <c r="A146" t="s">
         <v>241</v>
       </c>
@@ -4372,7 +4372,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:6">
       <c r="A147" t="s">
         <v>243</v>
       </c>
@@ -4386,7 +4386,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:6">
       <c r="A148" t="s">
         <v>245</v>
       </c>
@@ -4400,7 +4400,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:6">
       <c r="A149" t="s">
         <v>247</v>
       </c>
@@ -4414,7 +4414,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:6">
       <c r="A150" t="s">
         <v>248</v>
       </c>
@@ -4431,7 +4431,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:6">
       <c r="A151" t="s">
         <v>251</v>
       </c>
@@ -4445,7 +4445,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:6">
       <c r="A152" t="s">
         <v>253</v>
       </c>
@@ -4459,7 +4459,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:6">
       <c r="A153" t="s">
         <v>254</v>
       </c>
@@ -4476,7 +4476,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:6">
       <c r="A154" t="s">
         <v>256</v>
       </c>
@@ -4493,7 +4493,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:6">
       <c r="A155" t="s">
         <v>258</v>
       </c>
@@ -4510,7 +4510,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:6">
       <c r="A156" t="s">
         <v>260</v>
       </c>
@@ -4527,7 +4527,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:6">
       <c r="A157" t="s">
         <v>261</v>
       </c>
@@ -4544,7 +4544,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:6">
       <c r="A158" t="s">
         <v>263</v>
       </c>
@@ -4558,7 +4558,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:6">
       <c r="A159" t="s">
         <v>264</v>
       </c>
@@ -4575,7 +4575,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:6">
       <c r="A160" t="s">
         <v>265</v>
       </c>
@@ -4592,7 +4592,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:6">
       <c r="A161" t="s">
         <v>267</v>
       </c>
@@ -4609,7 +4609,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:6">
       <c r="A162" t="s">
         <v>268</v>
       </c>
@@ -4626,7 +4626,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:6">
       <c r="A163" t="s">
         <v>271</v>
       </c>
@@ -4643,7 +4643,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:6">
       <c r="A164" t="s">
         <v>273</v>
       </c>
@@ -4657,7 +4657,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:6">
       <c r="A165" t="s">
         <v>274</v>
       </c>
@@ -4674,7 +4674,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:6">
       <c r="A166" t="s">
         <v>275</v>
       </c>
@@ -4691,7 +4691,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:6">
       <c r="A167" t="s">
         <v>277</v>
       </c>
@@ -4708,7 +4708,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:6">
       <c r="A168" t="s">
         <v>279</v>
       </c>
@@ -4725,7 +4725,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:6">
       <c r="A169" t="s">
         <v>281</v>
       </c>
@@ -4742,7 +4742,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:6">
       <c r="A170" t="s">
         <v>283</v>
       </c>
@@ -4759,7 +4759,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:6">
       <c r="A171" t="s">
         <v>286</v>
       </c>
@@ -4776,7 +4776,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:6">
       <c r="A172" t="s">
         <v>288</v>
       </c>
@@ -4793,7 +4793,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="173" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:6">
       <c r="A173" t="s">
         <v>290</v>
       </c>
@@ -4807,7 +4807,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:6">
       <c r="A174" t="s">
         <v>292</v>
       </c>
@@ -4821,7 +4821,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:6">
       <c r="A175" t="s">
         <v>294</v>
       </c>
@@ -4838,7 +4838,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:6">
       <c r="A176" t="s">
         <v>297</v>
       </c>
@@ -4855,7 +4855,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:6">
       <c r="A177" t="s">
         <v>300</v>
       </c>
@@ -4872,7 +4872,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:6">
       <c r="A178" t="s">
         <v>301</v>
       </c>
@@ -4889,7 +4889,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="179" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:6">
       <c r="A179" t="s">
         <v>303</v>
       </c>
@@ -4906,7 +4906,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="180" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:6">
       <c r="A180" t="s">
         <v>305</v>
       </c>
@@ -4923,7 +4923,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="181" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:6">
       <c r="A181" t="s">
         <v>307</v>
       </c>
@@ -4940,7 +4940,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="182" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:6">
       <c r="A182" t="s">
         <v>309</v>
       </c>
@@ -4957,7 +4957,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="183" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:6">
       <c r="A183" t="s">
         <v>310</v>
       </c>
@@ -4971,7 +4971,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="184" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:6">
       <c r="A184" t="s">
         <v>311</v>
       </c>
@@ -4988,7 +4988,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="185" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:6">
       <c r="A185" t="s">
         <v>313</v>
       </c>
@@ -5005,7 +5005,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="186" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:6">
       <c r="A186" t="s">
         <v>314</v>
       </c>
@@ -5022,7 +5022,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="187" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:6">
       <c r="A187" t="s">
         <v>316</v>
       </c>
@@ -5036,7 +5036,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="188" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:6">
       <c r="A188" t="s">
         <v>317</v>
       </c>
@@ -5053,7 +5053,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="189" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:6">
       <c r="A189" t="s">
         <v>319</v>
       </c>
@@ -5070,7 +5070,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="190" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:6">
       <c r="A190" t="s">
         <v>320</v>
       </c>
@@ -5087,7 +5087,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="191" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:6">
       <c r="A191" t="s">
         <v>321</v>
       </c>
@@ -5104,7 +5104,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="192" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:6">
       <c r="A192" t="s">
         <v>323</v>
       </c>
@@ -5121,7 +5121,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="193" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:6">
       <c r="A193" t="s">
         <v>325</v>
       </c>
@@ -5138,7 +5138,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="194" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:6">
       <c r="A194" t="s">
         <v>327</v>
       </c>
@@ -5155,7 +5155,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="195" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:6">
       <c r="A195" t="s">
         <v>329</v>
       </c>
@@ -5169,7 +5169,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="196" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:6">
       <c r="A196" t="s">
         <v>331</v>
       </c>
@@ -5183,7 +5183,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="197" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:6">
       <c r="A197" t="s">
         <v>333</v>
       </c>
@@ -5200,7 +5200,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="198" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:6">
       <c r="A198" t="s">
         <v>335</v>
       </c>
@@ -5217,7 +5217,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="199" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:6">
       <c r="A199" t="s">
         <v>337</v>
       </c>
@@ -5231,7 +5231,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="200" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:6">
       <c r="A200" t="s">
         <v>339</v>
       </c>
@@ -5248,7 +5248,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="201" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:6">
       <c r="A201" t="s">
         <v>341</v>
       </c>
@@ -5262,7 +5262,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="202" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:6">
       <c r="A202" t="s">
         <v>343</v>
       </c>
@@ -5279,7 +5279,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="203" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:6">
       <c r="A203" t="s">
         <v>345</v>
       </c>
@@ -5296,7 +5296,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="204" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:6">
       <c r="A204" t="s">
         <v>347</v>
       </c>
@@ -5313,7 +5313,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="205" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:6">
       <c r="A205" t="s">
         <v>348</v>
       </c>
@@ -5327,7 +5327,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="206" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:6">
       <c r="A206" t="s">
         <v>349</v>
       </c>
@@ -5341,7 +5341,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="207" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:6">
       <c r="A207" t="s">
         <v>350</v>
       </c>
@@ -5358,7 +5358,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="208" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:6">
       <c r="A208" t="s">
         <v>352</v>
       </c>
@@ -5375,7 +5375,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="209" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:6">
       <c r="A209" t="s">
         <v>354</v>
       </c>
@@ -5392,7 +5392,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="210" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:6">
       <c r="A210" t="s">
         <v>356</v>
       </c>
@@ -5409,7 +5409,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="211" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:6">
       <c r="A211" t="s">
         <v>358</v>
       </c>
@@ -5426,7 +5426,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="212" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:6">
       <c r="A212" t="s">
         <v>359</v>
       </c>
@@ -5440,7 +5440,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="213" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:6">
       <c r="A213" t="s">
         <v>360</v>
       </c>
@@ -5457,7 +5457,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="214" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:6">
       <c r="A214" t="s">
         <v>362</v>
       </c>
@@ -5471,7 +5471,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="215" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:6">
       <c r="A215" t="s">
         <v>363</v>
       </c>
@@ -5485,7 +5485,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="216" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:6">
       <c r="A216" t="s">
         <v>365</v>
       </c>
@@ -5499,7 +5499,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="217" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:6">
       <c r="A217" t="s">
         <v>367</v>
       </c>
@@ -5516,7 +5516,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="218" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:6">
       <c r="A218" t="s">
         <v>369</v>
       </c>
@@ -5533,7 +5533,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="219" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:6">
       <c r="A219" t="s">
         <v>371</v>
       </c>
@@ -5547,7 +5547,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="220" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:6">
       <c r="A220" t="s">
         <v>372</v>
       </c>
@@ -5564,7 +5564,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="221" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:6">
       <c r="A221" t="s">
         <v>374</v>
       </c>
@@ -5581,7 +5581,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="222" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:6">
       <c r="A222" t="s">
         <v>375</v>
       </c>
@@ -5595,7 +5595,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="223" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:6">
       <c r="A223" t="s">
         <v>376</v>
       </c>
@@ -5612,7 +5612,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="224" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:6">
       <c r="A224" t="s">
         <v>377</v>
       </c>
@@ -5629,7 +5629,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="225" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:6">
       <c r="A225" t="s">
         <v>379</v>
       </c>
@@ -5646,7 +5646,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="226" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:6">
       <c r="A226" t="s">
         <v>381</v>
       </c>
@@ -5663,7 +5663,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="227" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:6">
       <c r="A227" t="s">
         <v>383</v>
       </c>
@@ -5677,7 +5677,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="228" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:6">
       <c r="A228" t="s">
         <v>384</v>
       </c>
@@ -5691,7 +5691,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="229" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:6">
       <c r="A229" t="s">
         <v>386</v>
       </c>
@@ -5708,7 +5708,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="230" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:6">
       <c r="A230" t="s">
         <v>388</v>
       </c>
@@ -5725,7 +5725,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="231" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:6">
       <c r="A231" t="s">
         <v>390</v>
       </c>
@@ -5739,7 +5739,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="232" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:6">
       <c r="A232" t="s">
         <v>391</v>
       </c>
@@ -5753,7 +5753,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="233" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:6">
       <c r="A233" t="s">
         <v>393</v>
       </c>
@@ -5770,7 +5770,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="234" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:6">
       <c r="A234" t="s">
         <v>395</v>
       </c>
@@ -5787,7 +5787,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="235" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:6">
       <c r="A235" t="s">
         <v>397</v>
       </c>
@@ -5804,7 +5804,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="236" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:6">
       <c r="A236" t="s">
         <v>399</v>
       </c>
@@ -5821,7 +5821,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="237" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:6">
       <c r="A237" t="s">
         <v>401</v>
       </c>
@@ -5838,7 +5838,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="238" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:6">
       <c r="A238" t="s">
         <v>403</v>
       </c>
@@ -5855,7 +5855,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="239" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:6">
       <c r="A239" t="s">
         <v>405</v>
       </c>
@@ -5869,7 +5869,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="240" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:6">
       <c r="A240" t="s">
         <v>407</v>
       </c>
@@ -5883,7 +5883,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="241" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:6">
       <c r="A241" t="s">
         <v>409</v>
       </c>
@@ -5900,7 +5900,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="242" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:6">
       <c r="A242" t="s">
         <v>410</v>
       </c>
@@ -5914,7 +5914,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="243" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:6">
       <c r="A243" t="s">
         <v>411</v>
       </c>
@@ -5928,7 +5928,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="244" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:6">
       <c r="A244" t="s">
         <v>412</v>
       </c>
@@ -5945,7 +5945,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="245" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:6">
       <c r="A245" t="s">
         <v>413</v>
       </c>
@@ -5962,7 +5962,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="246" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:6">
       <c r="A246" t="s">
         <v>414</v>
       </c>
@@ -5979,7 +5979,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="247" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:6">
       <c r="A247" t="s">
         <v>415</v>
       </c>
@@ -5996,7 +5996,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="248" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:6">
       <c r="A248" t="s">
         <v>418</v>
       </c>
@@ -6013,7 +6013,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="249" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:6">
       <c r="A249" t="s">
         <v>419</v>
       </c>
@@ -6027,7 +6027,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="250" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:6">
       <c r="A250" t="s">
         <v>420</v>
       </c>
@@ -6041,7 +6041,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="251" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:6">
       <c r="A251" t="s">
         <v>421</v>
       </c>
@@ -6055,7 +6055,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="252" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:6">
       <c r="A252" t="s">
         <v>422</v>
       </c>
@@ -6072,7 +6072,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="253" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:6">
       <c r="A253" t="s">
         <v>424</v>
       </c>
@@ -6089,7 +6089,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="254" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:6">
       <c r="A254" t="s">
         <v>426</v>
       </c>
@@ -6106,7 +6106,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="255" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:6">
       <c r="A255" t="s">
         <v>428</v>
       </c>
@@ -6120,7 +6120,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="256" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:6">
       <c r="A256" t="s">
         <v>429</v>
       </c>
@@ -6137,7 +6137,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="257" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:6">
       <c r="A257" t="s">
         <v>430</v>
       </c>
@@ -6151,7 +6151,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="258" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:6">
       <c r="A258" t="s">
         <v>431</v>
       </c>
@@ -6165,7 +6165,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="259" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:6">
       <c r="A259" t="s">
         <v>432</v>
       </c>
@@ -6182,7 +6182,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="260" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:6">
       <c r="A260" t="s">
         <v>434</v>
       </c>
@@ -6199,7 +6199,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="261" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:6">
       <c r="A261" t="s">
         <v>435</v>
       </c>
@@ -6216,7 +6216,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="262" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:6">
       <c r="A262" t="s">
         <v>437</v>
       </c>
@@ -6230,7 +6230,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="263" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="263" spans="1:6">
       <c r="A263" t="s">
         <v>439</v>
       </c>
@@ -6244,7 +6244,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="264" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:6">
       <c r="A264" t="s">
         <v>441</v>
       </c>
@@ -6258,7 +6258,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="265" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="265" spans="1:6">
       <c r="A265" t="s">
         <v>443</v>
       </c>
@@ -6272,7 +6272,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="266" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="266" spans="1:6">
       <c r="A266" t="s">
         <v>444</v>
       </c>
@@ -6286,7 +6286,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="267" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:6">
       <c r="A267" t="s">
         <v>445</v>
       </c>
@@ -6300,7 +6300,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="268" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:6">
       <c r="A268" t="s">
         <v>446</v>
       </c>
@@ -6314,7 +6314,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="269" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:6">
       <c r="A269" t="s">
         <v>447</v>
       </c>
@@ -6328,7 +6328,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="270" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:6">
       <c r="A270" t="s">
         <v>448</v>
       </c>
@@ -6345,7 +6345,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="271" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:6">
       <c r="A271" t="s">
         <v>450</v>
       </c>
@@ -6362,7 +6362,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="272" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:6">
       <c r="A272" t="s">
         <v>452</v>
       </c>
@@ -6376,7 +6376,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="273" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:6">
       <c r="A273" t="s">
         <v>453</v>
       </c>
@@ -6393,7 +6393,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="274" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:6">
       <c r="A274" t="s">
         <v>455</v>
       </c>
@@ -6407,7 +6407,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="275" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="275" spans="1:6">
       <c r="A275" t="s">
         <v>456</v>
       </c>
@@ -6421,7 +6421,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="276" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="276" spans="1:6">
       <c r="A276" t="s">
         <v>458</v>
       </c>
@@ -6435,7 +6435,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="277" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="277" spans="1:6">
       <c r="A277" t="s">
         <v>460</v>
       </c>
@@ -6449,7 +6449,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="278" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:6">
       <c r="A278" t="s">
         <v>462</v>
       </c>
@@ -6463,7 +6463,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="279" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:6">
       <c r="A279" t="s">
         <v>463</v>
       </c>
@@ -6477,7 +6477,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="280" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:6">
       <c r="A280" t="s">
         <v>464</v>
       </c>
@@ -6494,7 +6494,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="281" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="281" spans="1:6">
       <c r="A281" t="s">
         <v>466</v>
       </c>
@@ -6511,7 +6511,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="282" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:6">
       <c r="A282" t="s">
         <v>467</v>
       </c>
@@ -6525,7 +6525,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="283" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:6">
       <c r="A283" t="s">
         <v>468</v>
       </c>
@@ -6542,7 +6542,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="284" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:6">
       <c r="A284" t="s">
         <v>469</v>
       </c>
@@ -6559,7 +6559,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="285" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:6">
       <c r="A285" t="s">
         <v>470</v>
       </c>
@@ -6576,7 +6576,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="286" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:6">
       <c r="A286" t="s">
         <v>472</v>
       </c>
@@ -6593,7 +6593,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="287" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:6">
       <c r="A287" t="s">
         <v>474</v>
       </c>
@@ -6610,7 +6610,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="288" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:6">
       <c r="A288" t="s">
         <v>475</v>
       </c>
@@ -6627,7 +6627,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="289" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:6">
       <c r="A289" t="s">
         <v>477</v>
       </c>
@@ -6644,7 +6644,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="290" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:6">
       <c r="A290" t="s">
         <v>478</v>
       </c>
@@ -6661,7 +6661,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="291" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="291" spans="1:6">
       <c r="A291" t="s">
         <v>479</v>
       </c>
@@ -6678,7 +6678,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="292" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="292" spans="1:6">
       <c r="A292" t="s">
         <v>480</v>
       </c>
@@ -6695,7 +6695,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="293" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:6">
       <c r="A293" t="s">
         <v>482</v>
       </c>
@@ -6712,7 +6712,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="294" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="294" spans="1:6">
       <c r="A294" t="s">
         <v>484</v>
       </c>
@@ -6729,7 +6729,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="295" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="295" spans="1:6">
       <c r="A295" t="s">
         <v>486</v>
       </c>
@@ -6746,7 +6746,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="296" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:6">
       <c r="A296" t="s">
         <v>488</v>
       </c>
@@ -6763,7 +6763,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="297" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="297" spans="1:6">
       <c r="A297" t="s">
         <v>489</v>
       </c>
@@ -6780,7 +6780,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="298" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="298" spans="1:6">
       <c r="A298" t="s">
         <v>491</v>
       </c>
@@ -6797,7 +6797,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="299" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="299" spans="1:6">
       <c r="A299" t="s">
         <v>492</v>
       </c>
@@ -6814,7 +6814,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="300" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="300" spans="1:6">
       <c r="A300" t="s">
         <v>550</v>
       </c>
@@ -6825,7 +6825,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="301" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="301" spans="1:6">
       <c r="A301" t="s">
         <v>549</v>
       </c>
@@ -6836,7 +6836,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="302" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="302" spans="1:6">
       <c r="A302" t="s">
         <v>548</v>
       </c>
@@ -6847,18 +6847,18 @@
         <v>493</v>
       </c>
     </row>
-    <row r="303" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="303" spans="1:6">
       <c r="A303" t="s">
         <v>547</v>
       </c>
       <c r="C303" t="s">
-        <v>552</v>
+        <v>554</v>
       </c>
       <c r="F303" t="s">
         <v>493</v>
       </c>
     </row>
-    <row r="304" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="304" spans="1:6">
       <c r="A304" t="s">
         <v>546</v>
       </c>
@@ -6869,7 +6869,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="305" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="305" spans="1:6">
       <c r="A305" t="s">
         <v>545</v>
       </c>
@@ -6880,7 +6880,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="306" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="306" spans="1:6">
       <c r="A306" t="s">
         <v>544</v>
       </c>
@@ -6891,15 +6891,15 @@
         <v>493</v>
       </c>
     </row>
-    <row r="307" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="307" spans="1:6">
       <c r="A307" t="s">
         <v>551</v>
       </c>
       <c r="C307" t="s">
+        <v>552</v>
+      </c>
+      <c r="E307" t="s">
         <v>553</v>
-      </c>
-      <c r="E307" t="s">
-        <v>554</v>
       </c>
       <c r="F307" t="s">
         <v>493</v>
@@ -6914,9 +6914,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E009BBAC-B988-7C49-8FAA-EA75972BA821}">
   <dimension ref="A1:B18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.19921875" defaultRowHeight="15.6"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>146</v>
       </c>
@@ -6924,7 +6924,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2">
       <c r="A2" t="s">
         <v>155</v>
       </c>
@@ -6932,7 +6932,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>100</v>
       </c>
@@ -6940,7 +6940,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2">
       <c r="A4" t="s">
         <v>98</v>
       </c>
@@ -6948,7 +6948,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2">
       <c r="A5" t="s">
         <v>248</v>
       </c>
@@ -6956,7 +6956,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
         <v>251</v>
       </c>
@@ -6964,7 +6964,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2">
       <c r="A7" t="s">
         <v>176</v>
       </c>
@@ -6972,7 +6972,7 @@
         <v>495</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2">
       <c r="A8" t="s">
         <v>199</v>
       </c>
@@ -6980,7 +6980,7 @@
         <v>496</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2">
       <c r="A9" t="s">
         <v>239</v>
       </c>
@@ -6988,7 +6988,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2">
       <c r="A10" t="s">
         <v>245</v>
       </c>
@@ -6996,7 +6996,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2">
       <c r="A11" s="2" t="s">
         <v>235</v>
       </c>
@@ -7004,7 +7004,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2">
       <c r="A12" t="s">
         <v>237</v>
       </c>
@@ -7012,7 +7012,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2">
       <c r="A13" t="s">
         <v>241</v>
       </c>
@@ -7020,7 +7020,7 @@
         <v>497</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2">
       <c r="A14" t="s">
         <v>243</v>
       </c>
@@ -7028,7 +7028,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2">
       <c r="A15" t="s">
         <v>231</v>
       </c>
@@ -7036,7 +7036,7 @@
         <v>498</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2">
       <c r="A16" t="s">
         <v>233</v>
       </c>
@@ -7044,7 +7044,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2">
       <c r="A17" t="s">
         <v>500</v>
       </c>
@@ -7052,7 +7052,7 @@
         <v>501</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2">
       <c r="A18" t="s">
         <v>502</v>
       </c>

</xml_diff>

<commit_message>
Update to workflow for tables without deduplicate keys
</commit_message>
<xml_diff>
--- a/documentation/workflow/bc_bronze_workflow_mapping.xlsx
+++ b/documentation/workflow/bc_bronze_workflow_mapping.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fantasysuperkick/workspace/ccg/datawarehouse/documentation/workflow/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00093860-5EC9-0E42-A37A-DB25EA673172}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9852482F-FC3E-0D44-8C6D-82A28696BDA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="700" yWindow="500" windowWidth="28100" windowHeight="17500" xr2:uid="{2F7A961D-90EA-0F4A-9BBB-FA6BCAC4A400}"/>
+    <workbookView xWindow="-220" yWindow="600" windowWidth="28020" windowHeight="17400" xr2:uid="{2F7A961D-90EA-0F4A-9BBB-FA6BCAC4A400}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$C$1:$C$299</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$D$1:$D$307</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1431" uniqueCount="555">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1431" uniqueCount="558">
   <si>
     <t>3PLHeader</t>
   </si>
@@ -1596,9 +1596,6 @@
     <t>itemno, company, source_system</t>
   </si>
   <si>
-    <t>no, documentno, description, company, source_system</t>
-  </si>
-  <si>
     <t>startdate, company, source_system</t>
   </si>
   <si>
@@ -1611,9 +1608,6 @@
     <t>userid, company, source_system</t>
   </si>
   <si>
-    <t>documentno, description, no, company, source_system</t>
-  </si>
-  <si>
     <t>worksheetbatchname, company, source_system</t>
   </si>
   <si>
@@ -1623,9 +1617,6 @@
     <t>resourceno, company, source_system</t>
   </si>
   <si>
-    <t>documentno, lineno, no, description,, company, source_system</t>
-  </si>
-  <si>
     <t>journaltemplatename, lineno, company, source_system</t>
   </si>
   <si>
@@ -1705,6 +1696,24 @@
   </si>
   <si>
     <t>selltocustomerno, type, no, locationcode, postinggroup, unitofmeasure, shortcutdimension1code, customerpricegroup, jobno, orderno, billtocustomerno, genbuspostinggroup, genprodpostinggroup, vatcalculationtype, transactiontype, transportmethod, taxcategory, taxareacode, taxgroupcode, vatbuspostinggroup, vatprodpostinggroup, vatidentifier, jobtaskno, allocationaccountno, variantcode, bincode, unitofmeasurecode, depreciationbookcode, responsibilitycenter, itemcategorycode, customerdiscgroup, fundingbody</t>
+  </si>
+  <si>
+    <t>lineno, documentno, company, source_system</t>
+  </si>
+  <si>
+    <t>documentno, lineno, no, company, source_system</t>
+  </si>
+  <si>
+    <t>lineno,  company, source_system</t>
+  </si>
+  <si>
+    <t>documentno, lineno,  company, source_system</t>
+  </si>
+  <si>
+    <t>no, documentno, company, source_system</t>
+  </si>
+  <si>
+    <t>entryno, no, company, source_system</t>
   </si>
 </sst>
 </file>
@@ -2099,6 +2108,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4E95DFF8-97A2-F246-A8EF-BFAEB7CC069C}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:F307"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.1640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2117,7 +2127,7 @@
         <v>502</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>537</v>
+        <v>534</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>504</v>
@@ -2129,7 +2139,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -2146,7 +2156,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -2163,7 +2173,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>6</v>
       </c>
@@ -2177,7 +2187,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>8</v>
       </c>
@@ -2191,7 +2201,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -2208,7 +2218,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>13</v>
       </c>
@@ -2222,7 +2232,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>15</v>
       </c>
@@ -2239,7 +2249,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -2253,7 +2263,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>21</v>
       </c>
@@ -2270,7 +2280,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>22</v>
       </c>
@@ -2287,7 +2297,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>24</v>
       </c>
@@ -2304,7 +2314,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>26</v>
       </c>
@@ -2321,7 +2331,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>28</v>
       </c>
@@ -2338,7 +2348,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -2355,7 +2365,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>35</v>
       </c>
@@ -2369,7 +2379,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>36</v>
       </c>
@@ -2386,7 +2396,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>39</v>
       </c>
@@ -2400,7 +2410,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>42</v>
       </c>
@@ -2417,7 +2427,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>44</v>
       </c>
@@ -2434,7 +2444,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>46</v>
       </c>
@@ -2451,7 +2461,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>47</v>
       </c>
@@ -2468,7 +2478,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>49</v>
       </c>
@@ -2485,7 +2495,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>52</v>
       </c>
@@ -2499,7 +2509,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>53</v>
       </c>
@@ -2516,7 +2526,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>56</v>
       </c>
@@ -2533,7 +2543,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>58</v>
       </c>
@@ -2547,7 +2557,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>59</v>
       </c>
@@ -2569,7 +2579,7 @@
         <v>61</v>
       </c>
       <c r="C29" t="s">
-        <v>518</v>
+        <v>556</v>
       </c>
       <c r="E29" t="s">
         <v>62</v>
@@ -2578,7 +2588,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>63</v>
       </c>
@@ -2595,7 +2605,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>64</v>
       </c>
@@ -2612,12 +2622,12 @@
         <v>492</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>67</v>
       </c>
       <c r="C32" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="D32" t="s">
         <v>7</v>
@@ -2626,7 +2636,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>68</v>
       </c>
@@ -2643,7 +2653,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>69</v>
       </c>
@@ -2660,12 +2670,12 @@
         <v>492</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>72</v>
       </c>
       <c r="C35" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="D35" t="s">
         <v>7</v>
@@ -2674,7 +2684,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>73</v>
       </c>
@@ -2688,7 +2698,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>74</v>
       </c>
@@ -2705,7 +2715,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>77</v>
       </c>
@@ -2722,7 +2732,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>78</v>
       </c>
@@ -2736,7 +2746,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>80</v>
       </c>
@@ -2753,7 +2763,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>82</v>
       </c>
@@ -2770,7 +2780,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>84</v>
       </c>
@@ -2787,7 +2797,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>86</v>
       </c>
@@ -2804,12 +2814,12 @@
         <v>492</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>90</v>
       </c>
       <c r="C44" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="D44" t="s">
         <v>7</v>
@@ -2818,12 +2828,12 @@
         <v>492</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>91</v>
       </c>
       <c r="C45" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="D45" t="s">
         <v>7</v>
@@ -2832,7 +2842,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>92</v>
       </c>
@@ -2846,7 +2856,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>93</v>
       </c>
@@ -2860,7 +2870,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>94</v>
       </c>
@@ -2874,7 +2884,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>95</v>
       </c>
@@ -2891,7 +2901,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>97</v>
       </c>
@@ -2922,7 +2932,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>100</v>
       </c>
@@ -2939,7 +2949,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>103</v>
       </c>
@@ -2953,7 +2963,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>104</v>
       </c>
@@ -2967,7 +2977,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>105</v>
       </c>
@@ -2981,7 +2991,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>106</v>
       </c>
@@ -3012,7 +3022,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>110</v>
       </c>
@@ -3029,7 +3039,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>112</v>
       </c>
@@ -3046,12 +3056,12 @@
         <v>492</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>113</v>
       </c>
       <c r="C60" t="s">
-        <v>536</v>
+        <v>533</v>
       </c>
       <c r="D60" t="s">
         <v>7</v>
@@ -3063,7 +3073,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>115</v>
       </c>
@@ -3093,13 +3103,13 @@
         <v>117</v>
       </c>
       <c r="C63" t="s">
-        <v>535</v>
+        <v>532</v>
       </c>
       <c r="F63" t="s">
         <v>492</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>118</v>
       </c>
@@ -3116,7 +3126,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>120</v>
       </c>
@@ -3133,7 +3143,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>122</v>
       </c>
@@ -3147,7 +3157,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>123</v>
       </c>
@@ -3161,12 +3171,12 @@
         <v>492</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>124</v>
       </c>
       <c r="C68" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="D68" t="s">
         <v>7</v>
@@ -3175,7 +3185,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>125</v>
       </c>
@@ -3192,12 +3202,12 @@
         <v>492</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>128</v>
       </c>
       <c r="C70" t="s">
-        <v>534</v>
+        <v>531</v>
       </c>
       <c r="D70" t="s">
         <v>7</v>
@@ -3206,7 +3216,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>129</v>
       </c>
@@ -3220,12 +3230,12 @@
         <v>492</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>130</v>
       </c>
       <c r="C72" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="D72" t="s">
         <v>17</v>
@@ -3242,7 +3252,7 @@
         <v>132</v>
       </c>
       <c r="C73" t="s">
-        <v>533</v>
+        <v>530</v>
       </c>
       <c r="E73" t="s">
         <v>133</v>
@@ -3265,7 +3275,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>136</v>
       </c>
@@ -3279,7 +3289,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>137</v>
       </c>
@@ -3293,7 +3303,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>138</v>
       </c>
@@ -3312,7 +3322,7 @@
         <v>139</v>
       </c>
       <c r="C78" t="s">
-        <v>415</v>
+        <v>552</v>
       </c>
       <c r="E78" t="s">
         <v>131</v>
@@ -3321,7 +3331,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>140</v>
       </c>
@@ -3338,7 +3348,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>142</v>
       </c>
@@ -3352,7 +3362,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>143</v>
       </c>
@@ -3366,7 +3376,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>144</v>
       </c>
@@ -3383,7 +3393,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>146</v>
       </c>
@@ -3400,7 +3410,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>149</v>
       </c>
@@ -3417,12 +3427,12 @@
         <v>492</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>151</v>
       </c>
       <c r="C85" t="s">
-        <v>532</v>
+        <v>529</v>
       </c>
       <c r="D85" t="s">
         <v>7</v>
@@ -3434,7 +3444,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>152</v>
       </c>
@@ -3451,7 +3461,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>154</v>
       </c>
@@ -3470,7 +3480,7 @@
         <v>155</v>
       </c>
       <c r="C88" t="s">
-        <v>70</v>
+        <v>515</v>
       </c>
       <c r="E88" t="s">
         <v>156</v>
@@ -3479,12 +3489,12 @@
         <v>493</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>157</v>
       </c>
       <c r="C89" t="s">
-        <v>531</v>
+        <v>528</v>
       </c>
       <c r="D89" t="s">
         <v>7</v>
@@ -3493,7 +3503,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>158</v>
       </c>
@@ -3510,7 +3520,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>159</v>
       </c>
@@ -3527,7 +3537,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>161</v>
       </c>
@@ -3544,7 +3554,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>163</v>
       </c>
@@ -3558,7 +3568,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>164</v>
       </c>
@@ -3575,7 +3585,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>166</v>
       </c>
@@ -3592,7 +3602,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>168</v>
       </c>
@@ -3606,7 +3616,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>169</v>
       </c>
@@ -3623,7 +3633,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>171</v>
       </c>
@@ -3637,7 +3647,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>172</v>
       </c>
@@ -3654,7 +3664,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>174</v>
       </c>
@@ -3668,7 +3678,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>175</v>
       </c>
@@ -3685,7 +3695,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>176</v>
       </c>
@@ -3713,7 +3723,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>179</v>
       </c>
@@ -3730,7 +3740,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>181</v>
       </c>
@@ -3747,12 +3757,12 @@
         <v>492</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>183</v>
       </c>
       <c r="C106" t="s">
-        <v>530</v>
+        <v>527</v>
       </c>
       <c r="D106" t="s">
         <v>7</v>
@@ -3761,7 +3771,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>184</v>
       </c>
@@ -3778,7 +3788,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>185</v>
       </c>
@@ -3795,7 +3805,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>187</v>
       </c>
@@ -3809,7 +3819,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>188</v>
       </c>
@@ -3823,7 +3833,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>189</v>
       </c>
@@ -3840,7 +3850,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>191</v>
       </c>
@@ -3854,7 +3864,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>192</v>
       </c>
@@ -3868,12 +3878,12 @@
         <v>492</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>193</v>
       </c>
       <c r="C114" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="D114" t="s">
         <v>7</v>
@@ -3885,7 +3895,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>195</v>
       </c>
@@ -3907,7 +3917,7 @@
         <v>197</v>
       </c>
       <c r="C116" t="s">
-        <v>528</v>
+        <v>525</v>
       </c>
       <c r="E116" t="s">
         <v>198</v>
@@ -3930,7 +3940,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>201</v>
       </c>
@@ -3947,7 +3957,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>204</v>
       </c>
@@ -3964,7 +3974,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>205</v>
       </c>
@@ -3981,7 +3991,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>207</v>
       </c>
@@ -3995,7 +4005,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>208</v>
       </c>
@@ -4012,7 +4022,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>210</v>
       </c>
@@ -4029,7 +4039,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>211</v>
       </c>
@@ -4046,7 +4056,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>212</v>
       </c>
@@ -4063,7 +4073,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>213</v>
       </c>
@@ -4080,7 +4090,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>214</v>
       </c>
@@ -4094,7 +4104,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>215</v>
       </c>
@@ -4108,7 +4118,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>216</v>
       </c>
@@ -4122,7 +4132,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>217</v>
       </c>
@@ -4136,7 +4146,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>218</v>
       </c>
@@ -4153,7 +4163,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>220</v>
       </c>
@@ -4170,7 +4180,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>222</v>
       </c>
@@ -4184,7 +4194,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>223</v>
       </c>
@@ -4201,12 +4211,12 @@
         <v>492</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>224</v>
       </c>
       <c r="C135" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="D135" t="s">
         <v>7</v>
@@ -4215,7 +4225,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>225</v>
       </c>
@@ -4229,7 +4239,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>226</v>
       </c>
@@ -4243,7 +4253,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>227</v>
       </c>
@@ -4257,7 +4267,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>228</v>
       </c>
@@ -4274,7 +4284,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>230</v>
       </c>
@@ -4307,7 +4317,7 @@
         <v>233</v>
       </c>
       <c r="C142" t="s">
-        <v>33</v>
+        <v>553</v>
       </c>
       <c r="E142" t="s">
         <v>234</v>
@@ -4335,7 +4345,7 @@
         <v>237</v>
       </c>
       <c r="C144" t="s">
-        <v>33</v>
+        <v>553</v>
       </c>
       <c r="E144" t="s">
         <v>238</v>
@@ -4377,10 +4387,10 @@
         <v>243</v>
       </c>
       <c r="C147" t="s">
-        <v>33</v>
+        <v>553</v>
       </c>
       <c r="E147" t="s">
-        <v>554</v>
+        <v>551</v>
       </c>
       <c r="F147" t="s">
         <v>492</v>
@@ -4391,7 +4401,7 @@
         <v>244</v>
       </c>
       <c r="C148" t="s">
-        <v>33</v>
+        <v>553</v>
       </c>
       <c r="E148" t="s">
         <v>245</v>
@@ -4400,7 +4410,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>246</v>
       </c>
@@ -4414,7 +4424,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>247</v>
       </c>
@@ -4436,7 +4446,7 @@
         <v>250</v>
       </c>
       <c r="C151" t="s">
-        <v>70</v>
+        <v>515</v>
       </c>
       <c r="E151" t="s">
         <v>251</v>
@@ -4445,7 +4455,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>252</v>
       </c>
@@ -4459,7 +4469,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>253</v>
       </c>
@@ -4476,7 +4486,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>255</v>
       </c>
@@ -4493,7 +4503,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>257</v>
       </c>
@@ -4510,7 +4520,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>259</v>
       </c>
@@ -4527,7 +4537,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>260</v>
       </c>
@@ -4544,7 +4554,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>262</v>
       </c>
@@ -4558,7 +4568,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>263</v>
       </c>
@@ -4575,7 +4585,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
         <v>264</v>
       </c>
@@ -4592,7 +4602,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
         <v>266</v>
       </c>
@@ -4609,7 +4619,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
         <v>267</v>
       </c>
@@ -4626,7 +4636,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
         <v>270</v>
       </c>
@@ -4643,7 +4653,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
         <v>272</v>
       </c>
@@ -4657,7 +4667,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
         <v>273</v>
       </c>
@@ -4674,7 +4684,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
         <v>274</v>
       </c>
@@ -4691,7 +4701,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
         <v>276</v>
       </c>
@@ -4708,7 +4718,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
         <v>278</v>
       </c>
@@ -4725,7 +4735,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
         <v>280</v>
       </c>
@@ -4742,7 +4752,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
         <v>282</v>
       </c>
@@ -4759,7 +4769,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="171" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
         <v>285</v>
       </c>
@@ -4776,7 +4786,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="172" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
         <v>287</v>
       </c>
@@ -4798,7 +4808,7 @@
         <v>289</v>
       </c>
       <c r="C173" t="s">
-        <v>14</v>
+        <v>88</v>
       </c>
       <c r="E173" t="s">
         <v>290</v>
@@ -4812,7 +4822,7 @@
         <v>291</v>
       </c>
       <c r="C174" t="s">
-        <v>268</v>
+        <v>554</v>
       </c>
       <c r="E174" t="s">
         <v>292</v>
@@ -4821,7 +4831,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
         <v>293</v>
       </c>
@@ -4838,7 +4848,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
         <v>296</v>
       </c>
@@ -4855,7 +4865,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>299</v>
       </c>
@@ -4872,7 +4882,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>300</v>
       </c>
@@ -4889,7 +4899,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="179" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>302</v>
       </c>
@@ -4906,7 +4916,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="180" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
         <v>304</v>
       </c>
@@ -4923,7 +4933,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="181" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
         <v>306</v>
       </c>
@@ -4940,7 +4950,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="182" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
         <v>308</v>
       </c>
@@ -4957,7 +4967,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="183" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
         <v>309</v>
       </c>
@@ -4971,7 +4981,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="184" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
         <v>310</v>
       </c>
@@ -4988,7 +4998,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="185" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
         <v>312</v>
       </c>
@@ -5005,7 +5015,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="186" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
         <v>313</v>
       </c>
@@ -5022,7 +5032,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="187" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
         <v>315</v>
       </c>
@@ -5036,7 +5046,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="188" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
         <v>316</v>
       </c>
@@ -5053,7 +5063,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="189" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
         <v>318</v>
       </c>
@@ -5070,7 +5080,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="190" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
         <v>319</v>
       </c>
@@ -5087,7 +5097,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="191" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
         <v>320</v>
       </c>
@@ -5104,7 +5114,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="192" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
         <v>322</v>
       </c>
@@ -5121,7 +5131,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="193" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
         <v>324</v>
       </c>
@@ -5138,7 +5148,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="194" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
         <v>326</v>
       </c>
@@ -5174,7 +5184,7 @@
         <v>330</v>
       </c>
       <c r="C196" t="s">
-        <v>527</v>
+        <v>553</v>
       </c>
       <c r="E196" t="s">
         <v>331</v>
@@ -5183,7 +5193,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="197" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
         <v>332</v>
       </c>
@@ -5200,7 +5210,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="198" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
         <v>334</v>
       </c>
@@ -5231,7 +5241,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="200" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
         <v>338</v>
       </c>
@@ -5253,7 +5263,7 @@
         <v>340</v>
       </c>
       <c r="C201" t="s">
-        <v>33</v>
+        <v>553</v>
       </c>
       <c r="E201" t="s">
         <v>341</v>
@@ -5262,7 +5272,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="202" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
         <v>342</v>
       </c>
@@ -5279,7 +5289,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="203" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
         <v>344</v>
       </c>
@@ -5296,7 +5306,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="204" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
         <v>346</v>
       </c>
@@ -5313,7 +5323,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="205" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
         <v>347</v>
       </c>
@@ -5327,7 +5337,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="206" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
         <v>348</v>
       </c>
@@ -5341,7 +5351,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="207" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
         <v>349</v>
       </c>
@@ -5358,7 +5368,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="208" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
         <v>351</v>
       </c>
@@ -5375,7 +5385,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="209" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
         <v>353</v>
       </c>
@@ -5392,7 +5402,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="210" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
         <v>355</v>
       </c>
@@ -5409,12 +5419,12 @@
         <v>492</v>
       </c>
     </row>
-    <row r="211" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
         <v>357</v>
       </c>
       <c r="C211" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
       <c r="D211" t="s">
         <v>7</v>
@@ -5426,7 +5436,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="212" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
         <v>358</v>
       </c>
@@ -5440,7 +5450,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="213" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
         <v>359</v>
       </c>
@@ -5457,7 +5467,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="214" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
         <v>361</v>
       </c>
@@ -5490,7 +5500,7 @@
         <v>364</v>
       </c>
       <c r="C216" t="s">
-        <v>33</v>
+        <v>553</v>
       </c>
       <c r="E216" t="s">
         <v>365</v>
@@ -5499,7 +5509,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="217" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A217" t="s">
         <v>366</v>
       </c>
@@ -5516,7 +5526,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="218" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A218" t="s">
         <v>368</v>
       </c>
@@ -5533,7 +5543,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="219" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A219" t="s">
         <v>370</v>
       </c>
@@ -5547,7 +5557,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="220" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A220" t="s">
         <v>371</v>
       </c>
@@ -5564,7 +5574,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="221" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A221" t="s">
         <v>373</v>
       </c>
@@ -5581,7 +5591,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="222" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A222" t="s">
         <v>374</v>
       </c>
@@ -5595,7 +5605,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="223" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A223" t="s">
         <v>375</v>
       </c>
@@ -5612,7 +5622,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="224" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A224" t="s">
         <v>376</v>
       </c>
@@ -5629,7 +5639,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="225" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A225" t="s">
         <v>378</v>
       </c>
@@ -5646,7 +5656,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="226" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A226" t="s">
         <v>380</v>
       </c>
@@ -5663,7 +5673,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="227" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A227" t="s">
         <v>382</v>
       </c>
@@ -5682,7 +5692,7 @@
         <v>383</v>
       </c>
       <c r="C228" t="s">
-        <v>75</v>
+        <v>552</v>
       </c>
       <c r="E228" t="s">
         <v>384</v>
@@ -5691,7 +5701,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="229" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A229" t="s">
         <v>385</v>
       </c>
@@ -5708,7 +5718,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="230" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A230" t="s">
         <v>387</v>
       </c>
@@ -5753,7 +5763,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="233" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A233" t="s">
         <v>392</v>
       </c>
@@ -5770,7 +5780,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="234" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A234" t="s">
         <v>394</v>
       </c>
@@ -5787,7 +5797,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="235" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A235" t="s">
         <v>396</v>
       </c>
@@ -5804,7 +5814,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="236" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A236" t="s">
         <v>398</v>
       </c>
@@ -5821,12 +5831,12 @@
         <v>492</v>
       </c>
     </row>
-    <row r="237" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A237" t="s">
         <v>400</v>
       </c>
       <c r="C237" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="D237" t="s">
         <v>7</v>
@@ -5838,7 +5848,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="238" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A238" t="s">
         <v>402</v>
       </c>
@@ -5874,7 +5884,7 @@
         <v>406</v>
       </c>
       <c r="C240" t="s">
-        <v>33</v>
+        <v>553</v>
       </c>
       <c r="E240" t="s">
         <v>407</v>
@@ -5883,7 +5893,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="241" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A241" t="s">
         <v>408</v>
       </c>
@@ -5900,7 +5910,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="242" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A242" t="s">
         <v>409</v>
       </c>
@@ -5914,7 +5924,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="243" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A243" t="s">
         <v>410</v>
       </c>
@@ -5928,7 +5938,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="244" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A244" t="s">
         <v>411</v>
       </c>
@@ -5945,7 +5955,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="245" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A245" t="s">
         <v>412</v>
       </c>
@@ -5962,7 +5972,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="246" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A246" t="s">
         <v>413</v>
       </c>
@@ -5979,7 +5989,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="247" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A247" t="s">
         <v>414</v>
       </c>
@@ -5996,7 +6006,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="248" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A248" t="s">
         <v>417</v>
       </c>
@@ -6013,7 +6023,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="249" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A249" t="s">
         <v>418</v>
       </c>
@@ -6027,7 +6037,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="250" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A250" t="s">
         <v>419</v>
       </c>
@@ -6041,7 +6051,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="251" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A251" t="s">
         <v>420</v>
       </c>
@@ -6055,7 +6065,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="252" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A252" t="s">
         <v>421</v>
       </c>
@@ -6072,7 +6082,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="253" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A253" t="s">
         <v>423</v>
       </c>
@@ -6089,7 +6099,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="254" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A254" t="s">
         <v>425</v>
       </c>
@@ -6106,7 +6116,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="255" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A255" t="s">
         <v>427</v>
       </c>
@@ -6120,7 +6130,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="256" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A256" t="s">
         <v>428</v>
       </c>
@@ -6137,7 +6147,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="257" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A257" t="s">
         <v>429</v>
       </c>
@@ -6151,7 +6161,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="258" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A258" t="s">
         <v>430</v>
       </c>
@@ -6165,7 +6175,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="259" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A259" t="s">
         <v>431</v>
       </c>
@@ -6182,7 +6192,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="260" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A260" t="s">
         <v>433</v>
       </c>
@@ -6199,7 +6209,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="261" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A261" t="s">
         <v>434</v>
       </c>
@@ -6235,7 +6245,7 @@
         <v>438</v>
       </c>
       <c r="C263" t="s">
-        <v>4</v>
+        <v>555</v>
       </c>
       <c r="E263" t="s">
         <v>439</v>
@@ -6263,7 +6273,7 @@
         <v>442</v>
       </c>
       <c r="C265" t="s">
-        <v>4</v>
+        <v>555</v>
       </c>
       <c r="E265" t="s">
         <v>439</v>
@@ -6291,7 +6301,7 @@
         <v>444</v>
       </c>
       <c r="C267" t="s">
-        <v>4</v>
+        <v>111</v>
       </c>
       <c r="E267" t="s">
         <v>439</v>
@@ -6300,7 +6310,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="268" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A268" t="s">
         <v>445</v>
       </c>
@@ -6314,7 +6324,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="269" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A269" t="s">
         <v>446</v>
       </c>
@@ -6328,7 +6338,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="270" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A270" t="s">
         <v>447</v>
       </c>
@@ -6345,12 +6355,12 @@
         <v>492</v>
       </c>
     </row>
-    <row r="271" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A271" t="s">
         <v>449</v>
       </c>
       <c r="C271" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="D271" t="s">
         <v>7</v>
@@ -6362,7 +6372,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="272" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="272" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A272" t="s">
         <v>451</v>
       </c>
@@ -6376,7 +6386,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="273" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A273" t="s">
         <v>452</v>
       </c>
@@ -6393,7 +6403,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="274" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="274" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A274" t="s">
         <v>454</v>
       </c>
@@ -6412,7 +6422,7 @@
         <v>455</v>
       </c>
       <c r="C275" t="s">
-        <v>523</v>
+        <v>557</v>
       </c>
       <c r="E275" t="s">
         <v>456</v>
@@ -6440,7 +6450,7 @@
         <v>459</v>
       </c>
       <c r="C277" t="s">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="E277" t="s">
         <v>460</v>
@@ -6449,7 +6459,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="278" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A278" t="s">
         <v>461</v>
       </c>
@@ -6463,7 +6473,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="279" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="279" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A279" t="s">
         <v>462</v>
       </c>
@@ -6477,7 +6487,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="280" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="280" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A280" t="s">
         <v>463</v>
       </c>
@@ -6494,7 +6504,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="281" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="281" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A281" t="s">
         <v>465</v>
       </c>
@@ -6511,7 +6521,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="282" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="282" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A282" t="s">
         <v>466</v>
       </c>
@@ -6525,7 +6535,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="283" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="283" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A283" t="s">
         <v>467</v>
       </c>
@@ -6542,12 +6552,12 @@
         <v>492</v>
       </c>
     </row>
-    <row r="284" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="284" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A284" t="s">
         <v>468</v>
       </c>
       <c r="C284" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="D284" t="s">
         <v>7</v>
@@ -6559,7 +6569,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="285" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="285" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A285" t="s">
         <v>469</v>
       </c>
@@ -6576,7 +6586,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="286" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="286" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A286" t="s">
         <v>471</v>
       </c>
@@ -6593,7 +6603,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="287" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="287" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A287" t="s">
         <v>473</v>
       </c>
@@ -6610,7 +6620,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="288" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="288" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A288" t="s">
         <v>474</v>
       </c>
@@ -6627,7 +6637,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="289" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="289" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A289" t="s">
         <v>476</v>
       </c>
@@ -6644,7 +6654,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="290" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="290" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A290" t="s">
         <v>477</v>
       </c>
@@ -6661,7 +6671,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="291" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="291" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A291" t="s">
         <v>478</v>
       </c>
@@ -6678,7 +6688,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="292" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="292" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A292" t="s">
         <v>479</v>
       </c>
@@ -6695,7 +6705,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="293" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="293" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A293" t="s">
         <v>481</v>
       </c>
@@ -6712,7 +6722,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="294" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="294" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A294" t="s">
         <v>483</v>
       </c>
@@ -6729,7 +6739,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="295" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="295" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A295" t="s">
         <v>485</v>
       </c>
@@ -6746,7 +6756,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="296" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="296" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A296" t="s">
         <v>487</v>
       </c>
@@ -6763,7 +6773,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="297" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="297" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A297" t="s">
         <v>488</v>
       </c>
@@ -6780,7 +6790,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="298" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="298" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A298" t="s">
         <v>490</v>
       </c>
@@ -6797,7 +6807,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="299" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="299" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A299" t="s">
         <v>491</v>
       </c>
@@ -6816,10 +6826,10 @@
     </row>
     <row r="300" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A300" t="s">
-        <v>549</v>
+        <v>546</v>
       </c>
       <c r="C300" t="s">
-        <v>538</v>
+        <v>535</v>
       </c>
       <c r="F300" t="s">
         <v>492</v>
@@ -6827,10 +6837,10 @@
     </row>
     <row r="301" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A301" t="s">
-        <v>548</v>
+        <v>545</v>
       </c>
       <c r="C301" t="s">
-        <v>539</v>
+        <v>536</v>
       </c>
       <c r="F301" t="s">
         <v>492</v>
@@ -6838,10 +6848,10 @@
     </row>
     <row r="302" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A302" t="s">
-        <v>547</v>
+        <v>544</v>
       </c>
       <c r="C302" t="s">
-        <v>540</v>
+        <v>537</v>
       </c>
       <c r="F302" t="s">
         <v>492</v>
@@ -6849,10 +6859,10 @@
     </row>
     <row r="303" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A303" t="s">
-        <v>546</v>
+        <v>543</v>
       </c>
       <c r="C303" t="s">
-        <v>553</v>
+        <v>550</v>
       </c>
       <c r="F303" t="s">
         <v>492</v>
@@ -6860,10 +6870,10 @@
     </row>
     <row r="304" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A304" t="s">
-        <v>545</v>
+        <v>542</v>
       </c>
       <c r="C304" t="s">
-        <v>541</v>
+        <v>538</v>
       </c>
       <c r="F304" t="s">
         <v>492</v>
@@ -6871,10 +6881,10 @@
     </row>
     <row r="305" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A305" t="s">
-        <v>544</v>
+        <v>541</v>
       </c>
       <c r="C305" t="s">
-        <v>529</v>
+        <v>526</v>
       </c>
       <c r="F305" t="s">
         <v>492</v>
@@ -6882,33 +6892,38 @@
     </row>
     <row r="306" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A306" t="s">
-        <v>543</v>
+        <v>540</v>
       </c>
       <c r="C306" t="s">
-        <v>542</v>
+        <v>539</v>
       </c>
       <c r="F306" t="s">
         <v>492</v>
       </c>
     </row>
-    <row r="307" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="307" spans="1:6" hidden="1" x14ac:dyDescent="0.2">
       <c r="A307" t="s">
-        <v>550</v>
+        <v>547</v>
       </c>
       <c r="C307" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="D307" t="s">
-        <v>551</v>
+        <v>548</v>
       </c>
       <c r="E307" t="s">
-        <v>552</v>
+        <v>549</v>
       </c>
       <c r="F307" t="s">
         <v>492</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="D1:D307" xr:uid="{4E95DFF8-97A2-F246-A8EF-BFAEB7CC069C}">
+    <filterColumn colId="0">
+      <filters blank="1"/>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>